<commit_message>
Fix dynamic stage updates when n_ext/n_scr/n_str change in INPUTS
- SOLVER col B section labels are now Excel formulas (IF on INPUTS refs)
  instead of hardcoded Python strings
- Added conditional formatting on SOLVER A:B columns so row colors
  (yellow/green/red) update automatically when stage counts change
- RESULTS loaded-organic now uses INDEX(SOLVER!AM, 4+n_ext) instead of
  hardcoded row 14
- RESULTS preg concentration uses INDEX(col, 4+n_ext+n_scr+1) so it
  always points to the first strip stage regardless of configuration
- Raff (stage 1) remains a direct reference since it never moves

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EhkumPhB8AaWL9a7c6F6zJ
</commit_message>
<xml_diff>
--- a/SX_Steady_State_Model.xlsx
+++ b/SX_Steady_State_Model.xlsx
@@ -136,12 +136,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -181,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -265,43 +265,31 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -313,13 +301,13 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -338,6 +326,29 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -1906,10 +1917,9 @@
       <c r="A5" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="30" t="inlineStr">
-        <is>
-          <t>Extraction</t>
-        </is>
+      <c r="B5" s="30">
+        <f>IF(A5&lt;=INPUTS!$B$5,"Extraction",IF(A5&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C5" s="31">
         <f>IF(A5&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A5&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -2068,10 +2078,9 @@
       <c r="A6" s="29" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="30" t="inlineStr">
-        <is>
-          <t>Extraction</t>
-        </is>
+      <c r="B6" s="30">
+        <f>IF(A6&lt;=INPUTS!$B$5,"Extraction",IF(A6&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C6" s="34">
         <f>IF(A6&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A6&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -2230,10 +2239,9 @@
       <c r="A7" s="29" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="30" t="inlineStr">
-        <is>
-          <t>Extraction</t>
-        </is>
+      <c r="B7" s="30">
+        <f>IF(A7&lt;=INPUTS!$B$5,"Extraction",IF(A7&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C7" s="31">
         <f>IF(A7&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A7&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -2392,10 +2400,9 @@
       <c r="A8" s="29" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="30" t="inlineStr">
-        <is>
-          <t>Extraction</t>
-        </is>
+      <c r="B8" s="30">
+        <f>IF(A8&lt;=INPUTS!$B$5,"Extraction",IF(A8&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C8" s="34">
         <f>IF(A8&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A8&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -2554,10 +2561,9 @@
       <c r="A9" s="29" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="30" t="inlineStr">
-        <is>
-          <t>Extraction</t>
-        </is>
+      <c r="B9" s="30">
+        <f>IF(A9&lt;=INPUTS!$B$5,"Extraction",IF(A9&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C9" s="31">
         <f>IF(A9&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A9&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -2716,10 +2722,9 @@
       <c r="A10" s="29" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="30" t="inlineStr">
-        <is>
-          <t>Extraction</t>
-        </is>
+      <c r="B10" s="30">
+        <f>IF(A10&lt;=INPUTS!$B$5,"Extraction",IF(A10&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C10" s="34">
         <f>IF(A10&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A10&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -2878,10 +2883,9 @@
       <c r="A11" s="29" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="30" t="inlineStr">
-        <is>
-          <t>Extraction</t>
-        </is>
+      <c r="B11" s="30">
+        <f>IF(A11&lt;=INPUTS!$B$5,"Extraction",IF(A11&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C11" s="31">
         <f>IF(A11&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A11&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -3040,10 +3044,9 @@
       <c r="A12" s="29" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="30" t="inlineStr">
-        <is>
-          <t>Extraction</t>
-        </is>
+      <c r="B12" s="30">
+        <f>IF(A12&lt;=INPUTS!$B$5,"Extraction",IF(A12&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C12" s="34">
         <f>IF(A12&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A12&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -3202,10 +3205,9 @@
       <c r="A13" s="29" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="30" t="inlineStr">
-        <is>
-          <t>Extraction</t>
-        </is>
+      <c r="B13" s="30">
+        <f>IF(A13&lt;=INPUTS!$B$5,"Extraction",IF(A13&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C13" s="31">
         <f>IF(A13&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A13&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -3364,10 +3366,9 @@
       <c r="A14" s="29" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="30" t="inlineStr">
-        <is>
-          <t>Extraction</t>
-        </is>
+      <c r="B14" s="30">
+        <f>IF(A14&lt;=INPUTS!$B$5,"Extraction",IF(A14&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C14" s="34">
         <f>IF(A14&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A14&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -3523,13 +3524,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="35" t="n">
+      <c r="A15" s="29" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="36" t="inlineStr">
-        <is>
-          <t>Scrub</t>
-        </is>
+      <c r="B15" s="30">
+        <f>IF(A15&lt;=INPUTS!$B$5,"Extraction",IF(A15&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C15" s="31">
         <f>IF(A15&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A15&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -3685,13 +3685,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="35" t="n">
+      <c r="A16" s="29" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="36" t="inlineStr">
-        <is>
-          <t>Scrub</t>
-        </is>
+      <c r="B16" s="30">
+        <f>IF(A16&lt;=INPUTS!$B$5,"Extraction",IF(A16&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C16" s="34">
         <f>IF(A16&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A16&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -3847,13 +3846,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="35" t="n">
+      <c r="A17" s="29" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="36" t="inlineStr">
-        <is>
-          <t>Scrub</t>
-        </is>
+      <c r="B17" s="30">
+        <f>IF(A17&lt;=INPUTS!$B$5,"Extraction",IF(A17&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C17" s="31">
         <f>IF(A17&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A17&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -4009,13 +4007,12 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="35" t="n">
+      <c r="A18" s="29" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="36" t="inlineStr">
-        <is>
-          <t>Scrub</t>
-        </is>
+      <c r="B18" s="30">
+        <f>IF(A18&lt;=INPUTS!$B$5,"Extraction",IF(A18&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C18" s="34">
         <f>IF(A18&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A18&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -4171,13 +4168,12 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="35" t="n">
+      <c r="A19" s="29" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="36" t="inlineStr">
-        <is>
-          <t>Scrub</t>
-        </is>
+      <c r="B19" s="30">
+        <f>IF(A19&lt;=INPUTS!$B$5,"Extraction",IF(A19&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C19" s="31">
         <f>IF(A19&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A19&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -4333,13 +4329,12 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="35" t="n">
+      <c r="A20" s="29" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="36" t="inlineStr">
-        <is>
-          <t>Scrub</t>
-        </is>
+      <c r="B20" s="30">
+        <f>IF(A20&lt;=INPUTS!$B$5,"Extraction",IF(A20&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C20" s="34">
         <f>IF(A20&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A20&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -4495,13 +4490,12 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="35" t="n">
+      <c r="A21" s="29" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="36" t="inlineStr">
-        <is>
-          <t>Scrub</t>
-        </is>
+      <c r="B21" s="30">
+        <f>IF(A21&lt;=INPUTS!$B$5,"Extraction",IF(A21&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C21" s="31">
         <f>IF(A21&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A21&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -4657,13 +4651,12 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="35" t="n">
+      <c r="A22" s="29" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="36" t="inlineStr">
-        <is>
-          <t>Scrub</t>
-        </is>
+      <c r="B22" s="30">
+        <f>IF(A22&lt;=INPUTS!$B$5,"Extraction",IF(A22&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C22" s="34">
         <f>IF(A22&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A22&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -4819,13 +4812,12 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="35" t="n">
+      <c r="A23" s="29" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="36" t="inlineStr">
-        <is>
-          <t>Scrub</t>
-        </is>
+      <c r="B23" s="30">
+        <f>IF(A23&lt;=INPUTS!$B$5,"Extraction",IF(A23&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C23" s="31">
         <f>IF(A23&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A23&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -4981,13 +4973,12 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="35" t="n">
+      <c r="A24" s="29" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="36" t="inlineStr">
-        <is>
-          <t>Scrub</t>
-        </is>
+      <c r="B24" s="30">
+        <f>IF(A24&lt;=INPUTS!$B$5,"Extraction",IF(A24&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C24" s="34">
         <f>IF(A24&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A24&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -5143,13 +5134,12 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="37" t="n">
+      <c r="A25" s="29" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="38" t="inlineStr">
-        <is>
-          <t>Strip</t>
-        </is>
+      <c r="B25" s="30">
+        <f>IF(A25&lt;=INPUTS!$B$5,"Extraction",IF(A25&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C25" s="31">
         <f>IF(A25&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A25&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -5305,13 +5295,12 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="37" t="n">
+      <c r="A26" s="29" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="38" t="inlineStr">
-        <is>
-          <t>Strip</t>
-        </is>
+      <c r="B26" s="30">
+        <f>IF(A26&lt;=INPUTS!$B$5,"Extraction",IF(A26&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C26" s="34">
         <f>IF(A26&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A26&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -5467,13 +5456,12 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="37" t="n">
+      <c r="A27" s="29" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="38" t="inlineStr">
-        <is>
-          <t>Strip</t>
-        </is>
+      <c r="B27" s="30">
+        <f>IF(A27&lt;=INPUTS!$B$5,"Extraction",IF(A27&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C27" s="31">
         <f>IF(A27&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A27&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -5629,13 +5617,12 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="37" t="n">
+      <c r="A28" s="29" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="38" t="inlineStr">
-        <is>
-          <t>Strip</t>
-        </is>
+      <c r="B28" s="30">
+        <f>IF(A28&lt;=INPUTS!$B$5,"Extraction",IF(A28&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C28" s="34">
         <f>IF(A28&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A28&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -5791,13 +5778,12 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="37" t="n">
+      <c r="A29" s="29" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="38" t="inlineStr">
-        <is>
-          <t>Strip</t>
-        </is>
+      <c r="B29" s="30">
+        <f>IF(A29&lt;=INPUTS!$B$5,"Extraction",IF(A29&lt;=INPUTS!$B$5+INPUTS!$B$6,"Scrub","Strip"))</f>
+        <v/>
       </c>
       <c r="C29" s="31">
         <f>IF(A29&lt;=INPUTS!$B$5,INPUTS!$C$18*INPUTS!$B$8^INPUTS!$D$18,IF(A29&lt;=INPUTS!$B$5+INPUTS!$B$6,INPUTS!$C$18*INPUTS!$B$9^INPUTS!$D$18,INPUTS!$C$18*INPUTS!$B$10^INPUTS!$D$18))</f>
@@ -5963,6 +5949,17 @@
     <mergeCell ref="AI2:AL2"/>
     <mergeCell ref="A1:AN1"/>
   </mergeCells>
+  <conditionalFormatting sqref="A5:B29">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
+      <formula>$A5&gt;INPUTS!$B$5+INPUTS!$B$6</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1" stopIfTrue="0">
+      <formula>$A5&gt;INPUTS!$B$5</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2" stopIfTrue="0">
+      <formula>$A5&lt;=INPUTS!$B$5</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6002,16 +5999,16 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="39" t="inlineStr">
+      <c r="A4" s="35" t="inlineStr">
         <is>
           <t>Loaded Organic @ Ext Exit (g/L)</t>
         </is>
       </c>
-      <c r="B4" s="40">
-        <f>SOLVER!AM14</f>
-        <v/>
-      </c>
-      <c r="C4" s="41" t="inlineStr">
+      <c r="B4" s="36">
+        <f>INDEX(SOLVER!$AM:$AM,4+INPUTS!$B$5)</f>
+        <v/>
+      </c>
+      <c r="C4" s="37" t="inlineStr">
         <is>
           <t>[Target: 19.05]</t>
         </is>
@@ -6026,47 +6023,47 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="42" t="inlineStr">
+      <c r="A7" s="38" t="inlineStr">
         <is>
           <t>Element</t>
         </is>
       </c>
-      <c r="B7" s="42" t="inlineStr">
+      <c r="B7" s="38" t="inlineStr">
         <is>
           <t>Feed Conc.
 (g/L)</t>
         </is>
       </c>
-      <c r="C7" s="42" t="inlineStr">
+      <c r="C7" s="38" t="inlineStr">
         <is>
           <t>Raff Conc.
 (g/L)</t>
         </is>
       </c>
-      <c r="D7" s="42" t="inlineStr">
+      <c r="D7" s="38" t="inlineStr">
         <is>
           <t>Preg Conc.
 (g/L)</t>
         </is>
       </c>
-      <c r="E7" s="42" t="inlineStr">
+      <c r="E7" s="38" t="inlineStr">
         <is>
           <t>% Feed</t>
         </is>
       </c>
-      <c r="F7" s="42" t="inlineStr">
+      <c r="F7" s="38" t="inlineStr">
         <is>
           <t>% Raffinate</t>
         </is>
       </c>
-      <c r="G7" s="42" t="inlineStr">
+      <c r="G7" s="38" t="inlineStr">
         <is>
           <t>% Preg</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="43" t="inlineStr">
+      <c r="A8" s="39" t="inlineStr">
         <is>
           <t>Pr</t>
         </is>
@@ -6080,7 +6077,7 @@
         <v/>
       </c>
       <c r="D8" s="7">
-        <f>SOLVER!AI25</f>
+        <f>INDEX(SOLVER!$AI:$AI,4+INPUTS!$B$5+INPUTS!$B$6+1)</f>
         <v/>
       </c>
       <c r="E8" s="7">
@@ -6092,12 +6089,12 @@
         <v/>
       </c>
       <c r="G8" s="7">
-        <f>IF((SOLVER!AI25+SOLVER!AJ25+SOLVER!AK25+SOLVER!AL25)=0,0,SOLVER!AI25/(SOLVER!AI25+SOLVER!AJ25+SOLVER!AK25+SOLVER!AL25)*100)</f>
+        <f>IF((INDEX(SOLVER!$AI:$AI,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AJ:$AJ,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AK:$AK,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AL:$AL,4+INPUTS!$B$5+INPUTS!$B$6+1))=0,0,INDEX(SOLVER!$AI:$AI,4+INPUTS!$B$5+INPUTS!$B$6+1)/(INDEX(SOLVER!$AI:$AI,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AJ:$AJ,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AK:$AK,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AL:$AL,4+INPUTS!$B$5+INPUTS!$B$6+1))*100)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="44" t="inlineStr">
+      <c r="A9" s="40" t="inlineStr">
         <is>
           <t>Nd</t>
         </is>
@@ -6111,7 +6108,7 @@
         <v/>
       </c>
       <c r="D9" s="5">
-        <f>SOLVER!AJ25</f>
+        <f>INDEX(SOLVER!$AJ:$AJ,4+INPUTS!$B$5+INPUTS!$B$6+1)</f>
         <v/>
       </c>
       <c r="E9" s="5">
@@ -6123,12 +6120,12 @@
         <v/>
       </c>
       <c r="G9" s="5">
-        <f>IF((SOLVER!AI25+SOLVER!AJ25+SOLVER!AK25+SOLVER!AL25)=0,0,SOLVER!AJ25/(SOLVER!AI25+SOLVER!AJ25+SOLVER!AK25+SOLVER!AL25)*100)</f>
+        <f>IF((INDEX(SOLVER!$AI:$AI,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AJ:$AJ,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AK:$AK,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AL:$AL,4+INPUTS!$B$5+INPUTS!$B$6+1))=0,0,INDEX(SOLVER!$AJ:$AJ,4+INPUTS!$B$5+INPUTS!$B$6+1)/(INDEX(SOLVER!$AI:$AI,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AJ:$AJ,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AK:$AK,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AL:$AL,4+INPUTS!$B$5+INPUTS!$B$6+1))*100)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="43" t="inlineStr">
+      <c r="A10" s="39" t="inlineStr">
         <is>
           <t>Tb</t>
         </is>
@@ -6142,7 +6139,7 @@
         <v/>
       </c>
       <c r="D10" s="7">
-        <f>SOLVER!AK25</f>
+        <f>INDEX(SOLVER!$AK:$AK,4+INPUTS!$B$5+INPUTS!$B$6+1)</f>
         <v/>
       </c>
       <c r="E10" s="7">
@@ -6154,12 +6151,12 @@
         <v/>
       </c>
       <c r="G10" s="7">
-        <f>IF((SOLVER!AI25+SOLVER!AJ25+SOLVER!AK25+SOLVER!AL25)=0,0,SOLVER!AK25/(SOLVER!AI25+SOLVER!AJ25+SOLVER!AK25+SOLVER!AL25)*100)</f>
+        <f>IF((INDEX(SOLVER!$AI:$AI,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AJ:$AJ,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AK:$AK,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AL:$AL,4+INPUTS!$B$5+INPUTS!$B$6+1))=0,0,INDEX(SOLVER!$AK:$AK,4+INPUTS!$B$5+INPUTS!$B$6+1)/(INDEX(SOLVER!$AI:$AI,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AJ:$AJ,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AK:$AK,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AL:$AL,4+INPUTS!$B$5+INPUTS!$B$6+1))*100)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="44" t="inlineStr">
+      <c r="A11" s="40" t="inlineStr">
         <is>
           <t>Dy</t>
         </is>
@@ -6173,7 +6170,7 @@
         <v/>
       </c>
       <c r="D11" s="5">
-        <f>SOLVER!AL25</f>
+        <f>INDEX(SOLVER!$AL:$AL,4+INPUTS!$B$5+INPUTS!$B$6+1)</f>
         <v/>
       </c>
       <c r="E11" s="5">
@@ -6185,7 +6182,7 @@
         <v/>
       </c>
       <c r="G11" s="5">
-        <f>IF((SOLVER!AI25+SOLVER!AJ25+SOLVER!AK25+SOLVER!AL25)=0,0,SOLVER!AL25/(SOLVER!AI25+SOLVER!AJ25+SOLVER!AK25+SOLVER!AL25)*100)</f>
+        <f>IF((INDEX(SOLVER!$AI:$AI,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AJ:$AJ,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AK:$AK,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AL:$AL,4+INPUTS!$B$5+INPUTS!$B$6+1))=0,0,INDEX(SOLVER!$AL:$AL,4+INPUTS!$B$5+INPUTS!$B$6+1)/(INDEX(SOLVER!$AI:$AI,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AJ:$AJ,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AK:$AK,4+INPUTS!$B$5+INPUTS!$B$6+1)+INDEX(SOLVER!$AL:$AL,4+INPUTS!$B$5+INPUTS!$B$6+1))*100)</f>
         <v/>
       </c>
     </row>
@@ -6198,37 +6195,37 @@
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="42" t="inlineStr">
+      <c r="A15" s="38" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="B15" s="42" t="inlineStr">
+      <c r="B15" s="38" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C15" s="42" t="inlineStr">
+      <c r="C15" s="38" t="inlineStr">
         <is>
           <t>x_Pr</t>
         </is>
       </c>
-      <c r="D15" s="42" t="inlineStr">
+      <c r="D15" s="38" t="inlineStr">
         <is>
           <t>x_Nd</t>
         </is>
       </c>
-      <c r="E15" s="42" t="inlineStr">
+      <c r="E15" s="38" t="inlineStr">
         <is>
           <t>x_Tb</t>
         </is>
       </c>
-      <c r="F15" s="42" t="inlineStr">
+      <c r="F15" s="38" t="inlineStr">
         <is>
           <t>x_Dy</t>
         </is>
       </c>
-      <c r="G15" s="42" t="inlineStr">
+      <c r="G15" s="38" t="inlineStr">
         <is>
           <t>x_NdPr (grouped)</t>
         </is>
@@ -6245,31 +6242,31 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="45" t="n">
+      <c r="A16" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="45" t="inlineStr">
+      <c r="B16" s="41" t="inlineStr">
         <is>
           <t>Extraction</t>
         </is>
       </c>
-      <c r="C16" s="46">
+      <c r="C16" s="42">
         <f>SOLVER!AI5</f>
         <v/>
       </c>
-      <c r="D16" s="46">
+      <c r="D16" s="42">
         <f>SOLVER!AJ5</f>
         <v/>
       </c>
-      <c r="E16" s="46">
+      <c r="E16" s="42">
         <f>SOLVER!AK5</f>
         <v/>
       </c>
-      <c r="F16" s="46">
+      <c r="F16" s="42">
         <f>SOLVER!AL5</f>
         <v/>
       </c>
-      <c r="G16" s="47">
+      <c r="G16" s="43">
         <f>C16+D16</f>
         <v/>
       </c>
@@ -6307,7 +6304,7 @@
         <f>SOLVER!AL6</f>
         <v/>
       </c>
-      <c r="G17" s="47">
+      <c r="G17" s="43">
         <f>C17+D17</f>
         <v/>
       </c>
@@ -6321,31 +6318,31 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="45" t="n">
+      <c r="A18" s="41" t="n">
         <v>3</v>
       </c>
-      <c r="B18" s="45" t="inlineStr">
+      <c r="B18" s="41" t="inlineStr">
         <is>
           <t>Extraction</t>
         </is>
       </c>
-      <c r="C18" s="46">
+      <c r="C18" s="42">
         <f>SOLVER!AI7</f>
         <v/>
       </c>
-      <c r="D18" s="46">
+      <c r="D18" s="42">
         <f>SOLVER!AJ7</f>
         <v/>
       </c>
-      <c r="E18" s="46">
+      <c r="E18" s="42">
         <f>SOLVER!AK7</f>
         <v/>
       </c>
-      <c r="F18" s="46">
+      <c r="F18" s="42">
         <f>SOLVER!AL7</f>
         <v/>
       </c>
-      <c r="G18" s="47">
+      <c r="G18" s="43">
         <f>C18+D18</f>
         <v/>
       </c>
@@ -6383,7 +6380,7 @@
         <f>SOLVER!AL8</f>
         <v/>
       </c>
-      <c r="G19" s="47">
+      <c r="G19" s="43">
         <f>C19+D19</f>
         <v/>
       </c>
@@ -6397,31 +6394,31 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="45" t="n">
+      <c r="A20" s="41" t="n">
         <v>5</v>
       </c>
-      <c r="B20" s="45" t="inlineStr">
+      <c r="B20" s="41" t="inlineStr">
         <is>
           <t>Extraction</t>
         </is>
       </c>
-      <c r="C20" s="46">
+      <c r="C20" s="42">
         <f>SOLVER!AI9</f>
         <v/>
       </c>
-      <c r="D20" s="46">
+      <c r="D20" s="42">
         <f>SOLVER!AJ9</f>
         <v/>
       </c>
-      <c r="E20" s="46">
+      <c r="E20" s="42">
         <f>SOLVER!AK9</f>
         <v/>
       </c>
-      <c r="F20" s="46">
+      <c r="F20" s="42">
         <f>SOLVER!AL9</f>
         <v/>
       </c>
-      <c r="G20" s="47">
+      <c r="G20" s="43">
         <f>C20+D20</f>
         <v/>
       </c>
@@ -6459,7 +6456,7 @@
         <f>SOLVER!AL10</f>
         <v/>
       </c>
-      <c r="G21" s="47">
+      <c r="G21" s="43">
         <f>C21+D21</f>
         <v/>
       </c>
@@ -6473,31 +6470,31 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="45" t="n">
+      <c r="A22" s="41" t="n">
         <v>7</v>
       </c>
-      <c r="B22" s="45" t="inlineStr">
+      <c r="B22" s="41" t="inlineStr">
         <is>
           <t>Extraction</t>
         </is>
       </c>
-      <c r="C22" s="46">
+      <c r="C22" s="42">
         <f>SOLVER!AI11</f>
         <v/>
       </c>
-      <c r="D22" s="46">
+      <c r="D22" s="42">
         <f>SOLVER!AJ11</f>
         <v/>
       </c>
-      <c r="E22" s="46">
+      <c r="E22" s="42">
         <f>SOLVER!AK11</f>
         <v/>
       </c>
-      <c r="F22" s="46">
+      <c r="F22" s="42">
         <f>SOLVER!AL11</f>
         <v/>
       </c>
-      <c r="G22" s="47">
+      <c r="G22" s="43">
         <f>C22+D22</f>
         <v/>
       </c>
@@ -6535,7 +6532,7 @@
         <f>SOLVER!AL12</f>
         <v/>
       </c>
-      <c r="G23" s="47">
+      <c r="G23" s="43">
         <f>C23+D23</f>
         <v/>
       </c>
@@ -6549,31 +6546,31 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="45" t="n">
+      <c r="A24" s="41" t="n">
         <v>9</v>
       </c>
-      <c r="B24" s="45" t="inlineStr">
+      <c r="B24" s="41" t="inlineStr">
         <is>
           <t>Extraction</t>
         </is>
       </c>
-      <c r="C24" s="46">
+      <c r="C24" s="42">
         <f>SOLVER!AI13</f>
         <v/>
       </c>
-      <c r="D24" s="46">
+      <c r="D24" s="42">
         <f>SOLVER!AJ13</f>
         <v/>
       </c>
-      <c r="E24" s="46">
+      <c r="E24" s="42">
         <f>SOLVER!AK13</f>
         <v/>
       </c>
-      <c r="F24" s="46">
+      <c r="F24" s="42">
         <f>SOLVER!AL13</f>
         <v/>
       </c>
-      <c r="G24" s="47">
+      <c r="G24" s="43">
         <f>C24+D24</f>
         <v/>
       </c>
@@ -6611,7 +6608,7 @@
         <f>SOLVER!AL14</f>
         <v/>
       </c>
-      <c r="G25" s="47">
+      <c r="G25" s="43">
         <f>C25+D25</f>
         <v/>
       </c>
@@ -6625,31 +6622,31 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="48" t="n">
+      <c r="A26" s="44" t="n">
         <v>11</v>
       </c>
-      <c r="B26" s="48" t="inlineStr">
+      <c r="B26" s="44" t="inlineStr">
         <is>
           <t>Scrub</t>
         </is>
       </c>
-      <c r="C26" s="49">
+      <c r="C26" s="45">
         <f>SOLVER!AI15</f>
         <v/>
       </c>
-      <c r="D26" s="49">
+      <c r="D26" s="45">
         <f>SOLVER!AJ15</f>
         <v/>
       </c>
-      <c r="E26" s="49">
+      <c r="E26" s="45">
         <f>SOLVER!AK15</f>
         <v/>
       </c>
-      <c r="F26" s="49">
+      <c r="F26" s="45">
         <f>SOLVER!AL15</f>
         <v/>
       </c>
-      <c r="G26" s="47">
+      <c r="G26" s="43">
         <f>C26+D26</f>
         <v/>
       </c>
@@ -6687,7 +6684,7 @@
         <f>SOLVER!AL16</f>
         <v/>
       </c>
-      <c r="G27" s="47">
+      <c r="G27" s="43">
         <f>C27+D27</f>
         <v/>
       </c>
@@ -6701,31 +6698,31 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="48" t="n">
+      <c r="A28" s="44" t="n">
         <v>13</v>
       </c>
-      <c r="B28" s="48" t="inlineStr">
+      <c r="B28" s="44" t="inlineStr">
         <is>
           <t>Scrub</t>
         </is>
       </c>
-      <c r="C28" s="49">
+      <c r="C28" s="45">
         <f>SOLVER!AI17</f>
         <v/>
       </c>
-      <c r="D28" s="49">
+      <c r="D28" s="45">
         <f>SOLVER!AJ17</f>
         <v/>
       </c>
-      <c r="E28" s="49">
+      <c r="E28" s="45">
         <f>SOLVER!AK17</f>
         <v/>
       </c>
-      <c r="F28" s="49">
+      <c r="F28" s="45">
         <f>SOLVER!AL17</f>
         <v/>
       </c>
-      <c r="G28" s="47">
+      <c r="G28" s="43">
         <f>C28+D28</f>
         <v/>
       </c>
@@ -6763,7 +6760,7 @@
         <f>SOLVER!AL18</f>
         <v/>
       </c>
-      <c r="G29" s="47">
+      <c r="G29" s="43">
         <f>C29+D29</f>
         <v/>
       </c>
@@ -6777,31 +6774,31 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="48" t="n">
+      <c r="A30" s="44" t="n">
         <v>15</v>
       </c>
-      <c r="B30" s="48" t="inlineStr">
+      <c r="B30" s="44" t="inlineStr">
         <is>
           <t>Scrub</t>
         </is>
       </c>
-      <c r="C30" s="49">
+      <c r="C30" s="45">
         <f>SOLVER!AI19</f>
         <v/>
       </c>
-      <c r="D30" s="49">
+      <c r="D30" s="45">
         <f>SOLVER!AJ19</f>
         <v/>
       </c>
-      <c r="E30" s="49">
+      <c r="E30" s="45">
         <f>SOLVER!AK19</f>
         <v/>
       </c>
-      <c r="F30" s="49">
+      <c r="F30" s="45">
         <f>SOLVER!AL19</f>
         <v/>
       </c>
-      <c r="G30" s="47">
+      <c r="G30" s="43">
         <f>C30+D30</f>
         <v/>
       </c>
@@ -6839,7 +6836,7 @@
         <f>SOLVER!AL20</f>
         <v/>
       </c>
-      <c r="G31" s="47">
+      <c r="G31" s="43">
         <f>C31+D31</f>
         <v/>
       </c>
@@ -6853,31 +6850,31 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="48" t="n">
+      <c r="A32" s="44" t="n">
         <v>17</v>
       </c>
-      <c r="B32" s="48" t="inlineStr">
+      <c r="B32" s="44" t="inlineStr">
         <is>
           <t>Scrub</t>
         </is>
       </c>
-      <c r="C32" s="49">
+      <c r="C32" s="45">
         <f>SOLVER!AI21</f>
         <v/>
       </c>
-      <c r="D32" s="49">
+      <c r="D32" s="45">
         <f>SOLVER!AJ21</f>
         <v/>
       </c>
-      <c r="E32" s="49">
+      <c r="E32" s="45">
         <f>SOLVER!AK21</f>
         <v/>
       </c>
-      <c r="F32" s="49">
+      <c r="F32" s="45">
         <f>SOLVER!AL21</f>
         <v/>
       </c>
-      <c r="G32" s="47">
+      <c r="G32" s="43">
         <f>C32+D32</f>
         <v/>
       </c>
@@ -6915,7 +6912,7 @@
         <f>SOLVER!AL22</f>
         <v/>
       </c>
-      <c r="G33" s="47">
+      <c r="G33" s="43">
         <f>C33+D33</f>
         <v/>
       </c>
@@ -6929,31 +6926,31 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="48" t="n">
+      <c r="A34" s="44" t="n">
         <v>19</v>
       </c>
-      <c r="B34" s="48" t="inlineStr">
+      <c r="B34" s="44" t="inlineStr">
         <is>
           <t>Scrub</t>
         </is>
       </c>
-      <c r="C34" s="49">
+      <c r="C34" s="45">
         <f>SOLVER!AI23</f>
         <v/>
       </c>
-      <c r="D34" s="49">
+      <c r="D34" s="45">
         <f>SOLVER!AJ23</f>
         <v/>
       </c>
-      <c r="E34" s="49">
+      <c r="E34" s="45">
         <f>SOLVER!AK23</f>
         <v/>
       </c>
-      <c r="F34" s="49">
+      <c r="F34" s="45">
         <f>SOLVER!AL23</f>
         <v/>
       </c>
-      <c r="G34" s="47">
+      <c r="G34" s="43">
         <f>C34+D34</f>
         <v/>
       </c>
@@ -6991,7 +6988,7 @@
         <f>SOLVER!AL24</f>
         <v/>
       </c>
-      <c r="G35" s="47">
+      <c r="G35" s="43">
         <f>C35+D35</f>
         <v/>
       </c>
@@ -7005,31 +7002,31 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="50" t="n">
+      <c r="A36" s="46" t="n">
         <v>21</v>
       </c>
-      <c r="B36" s="50" t="inlineStr">
+      <c r="B36" s="46" t="inlineStr">
         <is>
           <t>Strip</t>
         </is>
       </c>
-      <c r="C36" s="51">
+      <c r="C36" s="47">
         <f>SOLVER!AI25</f>
         <v/>
       </c>
-      <c r="D36" s="51">
+      <c r="D36" s="47">
         <f>SOLVER!AJ25</f>
         <v/>
       </c>
-      <c r="E36" s="51">
+      <c r="E36" s="47">
         <f>SOLVER!AK25</f>
         <v/>
       </c>
-      <c r="F36" s="51">
+      <c r="F36" s="47">
         <f>SOLVER!AL25</f>
         <v/>
       </c>
-      <c r="G36" s="47">
+      <c r="G36" s="43">
         <f>C36+D36</f>
         <v/>
       </c>
@@ -7067,7 +7064,7 @@
         <f>SOLVER!AL26</f>
         <v/>
       </c>
-      <c r="G37" s="47">
+      <c r="G37" s="43">
         <f>C37+D37</f>
         <v/>
       </c>
@@ -7081,31 +7078,31 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="50" t="n">
+      <c r="A38" s="46" t="n">
         <v>23</v>
       </c>
-      <c r="B38" s="50" t="inlineStr">
+      <c r="B38" s="46" t="inlineStr">
         <is>
           <t>Strip</t>
         </is>
       </c>
-      <c r="C38" s="51">
+      <c r="C38" s="47">
         <f>SOLVER!AI27</f>
         <v/>
       </c>
-      <c r="D38" s="51">
+      <c r="D38" s="47">
         <f>SOLVER!AJ27</f>
         <v/>
       </c>
-      <c r="E38" s="51">
+      <c r="E38" s="47">
         <f>SOLVER!AK27</f>
         <v/>
       </c>
-      <c r="F38" s="51">
+      <c r="F38" s="47">
         <f>SOLVER!AL27</f>
         <v/>
       </c>
-      <c r="G38" s="47">
+      <c r="G38" s="43">
         <f>C38+D38</f>
         <v/>
       </c>
@@ -7143,7 +7140,7 @@
         <f>SOLVER!AL28</f>
         <v/>
       </c>
-      <c r="G39" s="47">
+      <c r="G39" s="43">
         <f>C39+D39</f>
         <v/>
       </c>
@@ -7157,31 +7154,31 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="50" t="n">
+      <c r="A40" s="46" t="n">
         <v>25</v>
       </c>
-      <c r="B40" s="50" t="inlineStr">
+      <c r="B40" s="46" t="inlineStr">
         <is>
           <t>Strip</t>
         </is>
       </c>
-      <c r="C40" s="51">
+      <c r="C40" s="47">
         <f>SOLVER!AI29</f>
         <v/>
       </c>
-      <c r="D40" s="51">
+      <c r="D40" s="47">
         <f>SOLVER!AJ29</f>
         <v/>
       </c>
-      <c r="E40" s="51">
+      <c r="E40" s="47">
         <f>SOLVER!AK29</f>
         <v/>
       </c>
-      <c r="F40" s="51">
+      <c r="F40" s="47">
         <f>SOLVER!AL29</f>
         <v/>
       </c>
-      <c r="G40" s="47">
+      <c r="G40" s="43">
         <f>C40+D40</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add Saponification & Organic Loading section below stage profile
Three-panel section starting at row 114:
- Panel 1 (Organic System Inputs): extractant dropdown (D2EHPA / Cyanex 801),
  diluent dropdown (Orfom / Kerosene), % extractant, NaOH wt% and flowrate;
  auto-calculates organic density, [extractant] in g/L and mol/L, [NaOH] mol/L
- Panel 2 (Saponification): loaded organic at ext exit via dynamic INDEX;
  theoretical NaOH required (3 mol/mol REE, Alind Eq.10); experimental
  saponification degree (mol NaOH supplied / mol extractant × 100)
- Panel 3 (Max Organic Loading): per-element max loading (stoichiometric 1/3
  capacity), feed-weighted mixed-REE max, current vs max utilization %

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SX_Steady_State_Model.xlsx
+++ b/SX_Steady_State_Model.xlsx
@@ -16,11 +16,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -131,8 +132,36 @@
       <color rgb="000D47A1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="002E4057"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00757575"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002E4057"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -209,6 +238,11 @@
         <fgColor rgb="00E8F5E9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F7FA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -264,7 +298,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -373,6 +407,51 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="17" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="17" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1163,7 +1242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN72"/>
+  <dimension ref="A1:AN132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6814,24 +6893,688 @@
         <v/>
       </c>
     </row>
+    <row r="113" ht="12" customHeight="1"/>
+    <row r="114" ht="26" customHeight="1">
+      <c r="A114" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SAPONIFICATION  ·  ORGANIC LOADING  ·  REAGENT REQUIREMENTS</t>
+        </is>
+      </c>
+      <c r="E114" s="39" t="n"/>
+      <c r="J114" s="39" t="n"/>
+    </row>
+    <row r="115" ht="17" customHeight="1">
+      <c r="A115" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Organic System — Inputs</t>
+        </is>
+      </c>
+      <c r="E115" s="39" t="n"/>
+      <c r="F115" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Saponification Calculation</t>
+        </is>
+      </c>
+      <c r="J115" s="39" t="n"/>
+      <c r="K115" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Maximum Organic Loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="15" customHeight="1">
+      <c r="A116" s="41" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="B116" s="41" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C116" s="41" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D116" s="41" t="inlineStr"/>
+      <c r="E116" s="42" t="n"/>
+      <c r="F116" s="41" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="G116" s="41" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="H116" s="41" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="I116" s="41" t="inlineStr"/>
+      <c r="J116" s="42" t="n"/>
+      <c r="K116" s="41" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="L116" s="41" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="M116" s="41" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="N116" s="41" t="inlineStr"/>
+    </row>
+    <row r="117" ht="15" customHeight="1">
+      <c r="A117" s="43" t="inlineStr">
+        <is>
+          <t>Extractant</t>
+        </is>
+      </c>
+      <c r="B117" s="11" t="inlineStr">
+        <is>
+          <t>Cyanex 801</t>
+        </is>
+      </c>
+      <c r="C117" s="44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D117" s="45" t="n"/>
+      <c r="E117" s="39" t="n"/>
+      <c r="F117" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Loaded Organic at Extraction Exit</t>
+        </is>
+      </c>
+      <c r="J117" s="39" t="n"/>
+      <c r="K117" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Extractant Capacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="16" customHeight="1">
+      <c r="A118" s="43" t="inlineStr">
+        <is>
+          <t>Extractant  MW</t>
+        </is>
+      </c>
+      <c r="B118" s="47">
+        <f>IF(B117="D2EHPA",322.4,IF(B117="Cyanex 801",290.4,322.4))</f>
+        <v/>
+      </c>
+      <c r="C118" s="44" t="inlineStr">
+        <is>
+          <t>g/mol</t>
+        </is>
+      </c>
+      <c r="D118" s="45" t="n"/>
+      <c r="E118" s="39" t="n"/>
+      <c r="F118" s="43" t="inlineStr">
+        <is>
+          <t>y_Pr  (org. conc., ext exit)</t>
+        </is>
+      </c>
+      <c r="G118" s="32">
+        <f>INDEX($J:$J,19+$B$6)</f>
+        <v/>
+      </c>
+      <c r="H118" s="44" t="inlineStr">
+        <is>
+          <t>g/L org</t>
+        </is>
+      </c>
+      <c r="I118" s="45" t="n"/>
+      <c r="J118" s="39" t="n"/>
+      <c r="K118" s="43" t="inlineStr">
+        <is>
+          <t>Available capacity  [extractant / 3]</t>
+        </is>
+      </c>
+      <c r="L118" s="48">
+        <f>B124/3</f>
+        <v/>
+      </c>
+      <c r="M118" s="44" t="inlineStr">
+        <is>
+          <t>mol REE / L org</t>
+        </is>
+      </c>
+      <c r="N118" s="45" t="n"/>
+    </row>
+    <row r="119" ht="15" customHeight="1">
+      <c r="A119" s="43" t="inlineStr">
+        <is>
+          <t>Diluent</t>
+        </is>
+      </c>
+      <c r="B119" s="11" t="inlineStr">
+        <is>
+          <t>Orfom</t>
+        </is>
+      </c>
+      <c r="C119" s="44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D119" s="45" t="n"/>
+      <c r="E119" s="39" t="n"/>
+      <c r="F119" s="43" t="inlineStr">
+        <is>
+          <t>y_Nd  (org. conc., ext exit)</t>
+        </is>
+      </c>
+      <c r="G119" s="32">
+        <f>INDEX($R:$R,19+$B$6)</f>
+        <v/>
+      </c>
+      <c r="H119" s="44" t="inlineStr">
+        <is>
+          <t>g/L org</t>
+        </is>
+      </c>
+      <c r="I119" s="45" t="n"/>
+      <c r="J119" s="39" t="n"/>
+      <c r="K119" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Max Loading per Element  (if pure feed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="16" customHeight="1">
+      <c r="A120" s="43" t="inlineStr">
+        <is>
+          <t>Diluent density</t>
+        </is>
+      </c>
+      <c r="B120" s="48">
+        <f>IF(B119="Orfom",0.785,IF(B119="Kerosene",0.8,0.785))</f>
+        <v/>
+      </c>
+      <c r="C120" s="44" t="inlineStr">
+        <is>
+          <t>g/mL</t>
+        </is>
+      </c>
+      <c r="D120" s="45" t="n"/>
+      <c r="E120" s="39" t="n"/>
+      <c r="F120" s="43" t="inlineStr">
+        <is>
+          <t>y_Tb  (org. conc., ext exit)</t>
+        </is>
+      </c>
+      <c r="G120" s="32">
+        <f>INDEX($Z:$Z,19+$B$6)</f>
+        <v/>
+      </c>
+      <c r="H120" s="44" t="inlineStr">
+        <is>
+          <t>g/L org</t>
+        </is>
+      </c>
+      <c r="I120" s="45" t="n"/>
+      <c r="J120" s="39" t="n"/>
+      <c r="K120" s="43" t="inlineStr">
+        <is>
+          <t>Max loading — Pr  (pure Pr feed)</t>
+        </is>
+      </c>
+      <c r="L120" s="47">
+        <f>L118*140.91</f>
+        <v/>
+      </c>
+      <c r="M120" s="44" t="inlineStr">
+        <is>
+          <t>g/L org</t>
+        </is>
+      </c>
+      <c r="N120" s="45" t="n"/>
+    </row>
+    <row r="121" ht="16" customHeight="1">
+      <c r="A121" s="43" t="inlineStr">
+        <is>
+          <t>Organic density</t>
+        </is>
+      </c>
+      <c r="B121" s="48">
+        <f>B122/100*IF(B117="D2EHPA",0.975,0.87)+(1-B122/100)*B120</f>
+        <v/>
+      </c>
+      <c r="C121" s="44" t="inlineStr">
+        <is>
+          <t>g/mL</t>
+        </is>
+      </c>
+      <c r="D121" s="45" t="n"/>
+      <c r="E121" s="39" t="n"/>
+      <c r="F121" s="43" t="inlineStr">
+        <is>
+          <t>y_Dy  (org. conc., ext exit)</t>
+        </is>
+      </c>
+      <c r="G121" s="32">
+        <f>INDEX($AH:$AH,19+$B$6)</f>
+        <v/>
+      </c>
+      <c r="H121" s="44" t="inlineStr">
+        <is>
+          <t>g/L org</t>
+        </is>
+      </c>
+      <c r="I121" s="45" t="n"/>
+      <c r="J121" s="39" t="n"/>
+      <c r="K121" s="43" t="inlineStr">
+        <is>
+          <t>Max loading — Nd  (pure Nd feed)</t>
+        </is>
+      </c>
+      <c r="L121" s="47">
+        <f>L118*144.24</f>
+        <v/>
+      </c>
+      <c r="M121" s="44" t="inlineStr">
+        <is>
+          <t>g/L org</t>
+        </is>
+      </c>
+      <c r="N121" s="45" t="n"/>
+    </row>
+    <row r="122" ht="16" customHeight="1">
+      <c r="A122" s="43" t="inlineStr">
+        <is>
+          <t>% Extractant</t>
+        </is>
+      </c>
+      <c r="B122" s="49" t="n">
+        <v>10</v>
+      </c>
+      <c r="C122" s="44" t="inlineStr">
+        <is>
+          <t>vol %</t>
+        </is>
+      </c>
+      <c r="D122" s="45" t="n"/>
+      <c r="E122" s="39" t="n"/>
+      <c r="F122" s="50" t="inlineStr">
+        <is>
+          <t>Total loaded organic</t>
+        </is>
+      </c>
+      <c r="G122" s="51">
+        <f>G118+G119+G120+G121</f>
+        <v/>
+      </c>
+      <c r="H122" s="44" t="inlineStr">
+        <is>
+          <t>g/L org</t>
+        </is>
+      </c>
+      <c r="I122" s="45" t="n"/>
+      <c r="J122" s="39" t="n"/>
+      <c r="K122" s="43" t="inlineStr">
+        <is>
+          <t>Max loading — Tb  (pure Tb feed)</t>
+        </is>
+      </c>
+      <c r="L122" s="47">
+        <f>L118*158.93</f>
+        <v/>
+      </c>
+      <c r="M122" s="44" t="inlineStr">
+        <is>
+          <t>g/L org</t>
+        </is>
+      </c>
+      <c r="N122" s="45" t="n"/>
+    </row>
+    <row r="123" ht="15" customHeight="1">
+      <c r="A123" s="43" t="inlineStr">
+        <is>
+          <t>[Extractant]</t>
+        </is>
+      </c>
+      <c r="B123" s="47">
+        <f>B122/100*B121*1000</f>
+        <v/>
+      </c>
+      <c r="C123" s="44" t="inlineStr">
+        <is>
+          <t>g/L org</t>
+        </is>
+      </c>
+      <c r="D123" s="45" t="n"/>
+      <c r="E123" s="39" t="n"/>
+      <c r="F123" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Theoretical NaOH  (Alind Eq. 10 — 3 mol NaOH per mol REE³⁺)</t>
+        </is>
+      </c>
+      <c r="J123" s="39" t="n"/>
+      <c r="K123" s="43" t="inlineStr">
+        <is>
+          <t>Max loading — Dy  (pure Dy feed)</t>
+        </is>
+      </c>
+      <c r="L123" s="47">
+        <f>L118*162.5</f>
+        <v/>
+      </c>
+      <c r="M123" s="44" t="inlineStr">
+        <is>
+          <t>g/L org</t>
+        </is>
+      </c>
+      <c r="N123" s="45" t="n"/>
+    </row>
+    <row r="124" ht="15" customHeight="1">
+      <c r="A124" s="43" t="inlineStr">
+        <is>
+          <t>[Extractant]</t>
+        </is>
+      </c>
+      <c r="B124" s="48">
+        <f>IF(B118=0,0,B123/B118)</f>
+        <v/>
+      </c>
+      <c r="C124" s="44" t="inlineStr">
+        <is>
+          <t>mol/L org</t>
+        </is>
+      </c>
+      <c r="D124" s="45" t="n"/>
+      <c r="E124" s="39" t="n"/>
+      <c r="F124" s="43" t="inlineStr">
+        <is>
+          <t>NaOH required</t>
+        </is>
+      </c>
+      <c r="G124" s="48">
+        <f>3*$B$14*(G118/140.91+G119/144.24+G120/158.93+G121/162.5)</f>
+        <v/>
+      </c>
+      <c r="H124" s="44" t="inlineStr">
+        <is>
+          <t>mol / [O·time]</t>
+        </is>
+      </c>
+      <c r="I124" s="45" t="n"/>
+      <c r="J124" s="39" t="n"/>
+      <c r="K124" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Max Loading — Current Feed Composition</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="16" customHeight="1">
+      <c r="A125" s="43" t="inlineStr">
+        <is>
+          <t>NaOH concentration</t>
+        </is>
+      </c>
+      <c r="B125" s="49" t="n">
+        <v>20</v>
+      </c>
+      <c r="C125" s="44" t="inlineStr">
+        <is>
+          <t>wt %</t>
+        </is>
+      </c>
+      <c r="D125" s="45" t="n"/>
+      <c r="E125" s="39" t="n"/>
+      <c r="F125" s="43" t="inlineStr">
+        <is>
+          <t>NaOH solution flowrate</t>
+        </is>
+      </c>
+      <c r="G125" s="48">
+        <f>IF(B127=0,0,G124/B127)</f>
+        <v/>
+      </c>
+      <c r="H125" s="44" t="inlineStr">
+        <is>
+          <t>L soln / [O·time]</t>
+        </is>
+      </c>
+      <c r="I125" s="45" t="n"/>
+      <c r="J125" s="39" t="n"/>
+      <c r="K125" s="43" t="inlineStr">
+        <is>
+          <t>Avg REE MW  (feed-weighted)</t>
+        </is>
+      </c>
+      <c r="L125" s="52">
+        <f>IF(($M$6+$M$7+$M$8+$M$9)=0,144.24,($M$6*140.91+$M$7*144.24+$M$8*158.93+$M$9*162.5)/($M$6+$M$7+$M$8+$M$9))</f>
+        <v/>
+      </c>
+      <c r="M125" s="44" t="inlineStr">
+        <is>
+          <t>g/mol</t>
+        </is>
+      </c>
+      <c r="N125" s="45" t="n"/>
+    </row>
+    <row r="126" ht="16" customHeight="1">
+      <c r="A126" s="43" t="inlineStr">
+        <is>
+          <t>NaOH soln density</t>
+        </is>
+      </c>
+      <c r="B126" s="48">
+        <f>1+0.011*B125</f>
+        <v/>
+      </c>
+      <c r="C126" s="44" t="inlineStr">
+        <is>
+          <t>g/mL</t>
+        </is>
+      </c>
+      <c r="D126" s="45" t="n"/>
+      <c r="E126" s="39" t="n"/>
+      <c r="F126" s="43" t="inlineStr">
+        <is>
+          <t>Pure NaOH mass rate</t>
+        </is>
+      </c>
+      <c r="G126" s="48">
+        <f>G124*40.0/1000</f>
+        <v/>
+      </c>
+      <c r="H126" s="44" t="inlineStr">
+        <is>
+          <t>kg NaOH / [O·time]</t>
+        </is>
+      </c>
+      <c r="I126" s="45" t="n"/>
+      <c r="J126" s="39" t="n"/>
+      <c r="K126" s="50" t="inlineStr">
+        <is>
+          <t>Max loading — mixed REE</t>
+        </is>
+      </c>
+      <c r="L126" s="53">
+        <f>L118*L125</f>
+        <v/>
+      </c>
+      <c r="M126" s="44" t="inlineStr">
+        <is>
+          <t>g/L org</t>
+        </is>
+      </c>
+      <c r="N126" s="45" t="n"/>
+    </row>
+    <row r="127" ht="16" customHeight="1">
+      <c r="A127" s="43" t="inlineStr">
+        <is>
+          <t>[NaOH] solution</t>
+        </is>
+      </c>
+      <c r="B127" s="48">
+        <f>B125/100*B126*1000/40.0</f>
+        <v/>
+      </c>
+      <c r="C127" s="44" t="inlineStr">
+        <is>
+          <t>mol/L</t>
+        </is>
+      </c>
+      <c r="D127" s="45" t="n"/>
+      <c r="E127" s="39" t="n"/>
+      <c r="F127" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Experimental Saponification Degree</t>
+        </is>
+      </c>
+      <c r="J127" s="39" t="n"/>
+      <c r="K127" s="43" t="inlineStr">
+        <is>
+          <t>Current loaded organic  (from SOLVER)</t>
+        </is>
+      </c>
+      <c r="L127" s="54">
+        <f>INDEX($AM:$AM,19+$B$6)</f>
+        <v/>
+      </c>
+      <c r="M127" s="44" t="inlineStr">
+        <is>
+          <t>g/L org</t>
+        </is>
+      </c>
+      <c r="N127" s="45" t="n"/>
+    </row>
+    <row r="128" ht="16" customHeight="1">
+      <c r="A128" s="43" t="inlineStr">
+        <is>
+          <t>NaOH flowrate</t>
+        </is>
+      </c>
+      <c r="B128" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C128" s="44" t="inlineStr">
+        <is>
+          <t>same unit as O</t>
+        </is>
+      </c>
+      <c r="D128" s="45" t="n"/>
+      <c r="E128" s="39" t="n"/>
+      <c r="F128" s="43" t="inlineStr">
+        <is>
+          <t>mol NaOH supplied  [per time unit]</t>
+        </is>
+      </c>
+      <c r="G128" s="48">
+        <f>B128*B127</f>
+        <v/>
+      </c>
+      <c r="H128" s="44" t="inlineStr">
+        <is>
+          <t>mol / time</t>
+        </is>
+      </c>
+      <c r="I128" s="45" t="n"/>
+      <c r="J128" s="39" t="n"/>
+      <c r="K128" s="50" t="inlineStr">
+        <is>
+          <t>Loading utilization</t>
+        </is>
+      </c>
+      <c r="L128" s="53">
+        <f>IF(L126=0,0,L127/L126*100)</f>
+        <v/>
+      </c>
+      <c r="M128" s="44" t="inlineStr">
+        <is>
+          <t>%  of max capacity used</t>
+        </is>
+      </c>
+      <c r="N128" s="45" t="n"/>
+    </row>
+    <row r="129" ht="16" customHeight="1">
+      <c r="E129" s="39" t="n"/>
+      <c r="F129" s="43" t="inlineStr">
+        <is>
+          <t>mol D2EHPA/extr. in organic  [per time unit]</t>
+        </is>
+      </c>
+      <c r="G129" s="48">
+        <f>B124*$B$14</f>
+        <v/>
+      </c>
+      <c r="H129" s="44" t="inlineStr">
+        <is>
+          <t>mol / time</t>
+        </is>
+      </c>
+      <c r="I129" s="45" t="n"/>
+      <c r="J129" s="39" t="n"/>
+    </row>
+    <row r="130" ht="16" customHeight="1">
+      <c r="E130" s="39" t="n"/>
+      <c r="F130" s="50" t="inlineStr">
+        <is>
+          <t>SAPONIFICATION DEGREE</t>
+        </is>
+      </c>
+      <c r="G130" s="53">
+        <f>IF(G129=0,0,G128/G129*100)</f>
+        <v/>
+      </c>
+      <c r="H130" s="44" t="inlineStr">
+        <is>
+          <t>% saponified</t>
+        </is>
+      </c>
+      <c r="I130" s="45" t="n"/>
+      <c r="J130" s="39" t="n"/>
+    </row>
+    <row r="131" ht="16" customHeight="1">
+      <c r="E131" s="39" t="n"/>
+      <c r="J131" s="39" t="n"/>
+    </row>
+    <row r="132" ht="16" customHeight="1">
+      <c r="E132" s="39" t="n"/>
+      <c r="J132" s="39" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="29">
+    <mergeCell ref="K119:M119"/>
+    <mergeCell ref="A114:N114"/>
     <mergeCell ref="AI18:AL18"/>
     <mergeCell ref="Q2:T2"/>
+    <mergeCell ref="F115:I115"/>
+    <mergeCell ref="A115:D115"/>
     <mergeCell ref="A17:AN17"/>
     <mergeCell ref="S18:Z18"/>
     <mergeCell ref="E2:H2"/>
+    <mergeCell ref="K117:M117"/>
     <mergeCell ref="A47:I47"/>
     <mergeCell ref="F4:I4"/>
     <mergeCell ref="I2:L2"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="O4:P4"/>
+    <mergeCell ref="F117:H117"/>
     <mergeCell ref="K4:M4"/>
+    <mergeCell ref="F123:H123"/>
+    <mergeCell ref="K124:M124"/>
     <mergeCell ref="M2:P2"/>
     <mergeCell ref="A1:AN1"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="AA18:AH18"/>
+    <mergeCell ref="F127:H127"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="K115:N115"/>
     <mergeCell ref="AM18:AN18"/>
     <mergeCell ref="K18:R18"/>
     <mergeCell ref="C18:J18"/>
@@ -6847,6 +7590,14 @@
       <formula>$A20&lt;=$B$6</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="B117" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"D2EHPA,Cyanex 801"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Orfom,Kerosene"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix TDMA boundary: c=0 at last scrub stage (scrub and strip are separate aqueous circuits)
The c-coefficient at stage n_ext+n_scr was incorrectly coupling to the strip section
with SR/D_strip. Fresh scrub acid enters at stage n_ext+n_scr as an independent
boundary condition (same pattern as fresh strip acid entering at stage N=25 where c=0).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EhkumPhB8AaWL9a7c6F6zJ
</commit_message>
<xml_diff>
--- a/SX_Steady_State_Model.xlsx
+++ b/SX_Steady_State_Model.xlsx
@@ -2015,7 +2015,7 @@
         <v/>
       </c>
       <c r="F20" s="30">
-        <f>IF(A20&gt;$B$6+$B$7,$B$13/C21,IF(A20&gt;=$B$6,$B$13*$B$15/C21,($B$13*$B$15+$B$12)/C21))</f>
+        <f>IF(A20&gt;$B$6+$B$7,$B$13/C21,IF(A20=$B$6+$B$7,0,IF(A20&gt;=$B$6,$B$13*$B$15/C21,($B$13*$B$15+$B$12)/C21)))</f>
         <v/>
       </c>
       <c r="G20" s="30">
@@ -2047,7 +2047,7 @@
         <v/>
       </c>
       <c r="N20" s="30">
-        <f>IF(A20&gt;$B$6+$B$7,$B$13/K21,IF(A20&gt;=$B$6,$B$13*$B$15/K21,($B$13*$B$15+$B$12)/K21))</f>
+        <f>IF(A20&gt;$B$6+$B$7,$B$13/K21,IF(A20=$B$6+$B$7,0,IF(A20&gt;=$B$6,$B$13*$B$15/K21,($B$13*$B$15+$B$12)/K21)))</f>
         <v/>
       </c>
       <c r="O20" s="30">
@@ -2079,7 +2079,7 @@
         <v/>
       </c>
       <c r="V20" s="30">
-        <f>IF(A20&gt;$B$6+$B$7,$B$13/S21,IF(A20&gt;=$B$6,$B$13*$B$15/S21,($B$13*$B$15+$B$12)/S21))</f>
+        <f>IF(A20&gt;$B$6+$B$7,$B$13/S21,IF(A20=$B$6+$B$7,0,IF(A20&gt;=$B$6,$B$13*$B$15/S21,($B$13*$B$15+$B$12)/S21)))</f>
         <v/>
       </c>
       <c r="W20" s="30">
@@ -2111,7 +2111,7 @@
         <v/>
       </c>
       <c r="AD20" s="30">
-        <f>IF(A20&gt;$B$6+$B$7,$B$13/AA21,IF(A20&gt;=$B$6,$B$13*$B$15/AA21,($B$13*$B$15+$B$12)/AA21))</f>
+        <f>IF(A20&gt;$B$6+$B$7,$B$13/AA21,IF(A20=$B$6+$B$7,0,IF(A20&gt;=$B$6,$B$13*$B$15/AA21,($B$13*$B$15+$B$12)/AA21)))</f>
         <v/>
       </c>
       <c r="AE20" s="30">
@@ -2176,7 +2176,7 @@
         <v/>
       </c>
       <c r="F21" s="30">
-        <f>IF(A21&gt;$B$6+$B$7,$B$13/C22,IF(A21&gt;=$B$6,$B$13*$B$15/C22,($B$13*$B$15+$B$12)/C22))</f>
+        <f>IF(A21&gt;$B$6+$B$7,$B$13/C22,IF(A21=$B$6+$B$7,0,IF(A21&gt;=$B$6,$B$13*$B$15/C22,($B$13*$B$15+$B$12)/C22)))</f>
         <v/>
       </c>
       <c r="G21" s="30">
@@ -2208,7 +2208,7 @@
         <v/>
       </c>
       <c r="N21" s="30">
-        <f>IF(A21&gt;$B$6+$B$7,$B$13/K22,IF(A21&gt;=$B$6,$B$13*$B$15/K22,($B$13*$B$15+$B$12)/K22))</f>
+        <f>IF(A21&gt;$B$6+$B$7,$B$13/K22,IF(A21=$B$6+$B$7,0,IF(A21&gt;=$B$6,$B$13*$B$15/K22,($B$13*$B$15+$B$12)/K22)))</f>
         <v/>
       </c>
       <c r="O21" s="30">
@@ -2240,7 +2240,7 @@
         <v/>
       </c>
       <c r="V21" s="30">
-        <f>IF(A21&gt;$B$6+$B$7,$B$13/S22,IF(A21&gt;=$B$6,$B$13*$B$15/S22,($B$13*$B$15+$B$12)/S22))</f>
+        <f>IF(A21&gt;$B$6+$B$7,$B$13/S22,IF(A21=$B$6+$B$7,0,IF(A21&gt;=$B$6,$B$13*$B$15/S22,($B$13*$B$15+$B$12)/S22)))</f>
         <v/>
       </c>
       <c r="W21" s="30">
@@ -2272,7 +2272,7 @@
         <v/>
       </c>
       <c r="AD21" s="30">
-        <f>IF(A21&gt;$B$6+$B$7,$B$13/AA22,IF(A21&gt;=$B$6,$B$13*$B$15/AA22,($B$13*$B$15+$B$12)/AA22))</f>
+        <f>IF(A21&gt;$B$6+$B$7,$B$13/AA22,IF(A21=$B$6+$B$7,0,IF(A21&gt;=$B$6,$B$13*$B$15/AA22,($B$13*$B$15+$B$12)/AA22)))</f>
         <v/>
       </c>
       <c r="AE21" s="30">
@@ -2337,7 +2337,7 @@
         <v/>
       </c>
       <c r="F22" s="30">
-        <f>IF(A22&gt;$B$6+$B$7,$B$13/C23,IF(A22&gt;=$B$6,$B$13*$B$15/C23,($B$13*$B$15+$B$12)/C23))</f>
+        <f>IF(A22&gt;$B$6+$B$7,$B$13/C23,IF(A22=$B$6+$B$7,0,IF(A22&gt;=$B$6,$B$13*$B$15/C23,($B$13*$B$15+$B$12)/C23)))</f>
         <v/>
       </c>
       <c r="G22" s="30">
@@ -2369,7 +2369,7 @@
         <v/>
       </c>
       <c r="N22" s="30">
-        <f>IF(A22&gt;$B$6+$B$7,$B$13/K23,IF(A22&gt;=$B$6,$B$13*$B$15/K23,($B$13*$B$15+$B$12)/K23))</f>
+        <f>IF(A22&gt;$B$6+$B$7,$B$13/K23,IF(A22=$B$6+$B$7,0,IF(A22&gt;=$B$6,$B$13*$B$15/K23,($B$13*$B$15+$B$12)/K23)))</f>
         <v/>
       </c>
       <c r="O22" s="30">
@@ -2401,7 +2401,7 @@
         <v/>
       </c>
       <c r="V22" s="30">
-        <f>IF(A22&gt;$B$6+$B$7,$B$13/S23,IF(A22&gt;=$B$6,$B$13*$B$15/S23,($B$13*$B$15+$B$12)/S23))</f>
+        <f>IF(A22&gt;$B$6+$B$7,$B$13/S23,IF(A22=$B$6+$B$7,0,IF(A22&gt;=$B$6,$B$13*$B$15/S23,($B$13*$B$15+$B$12)/S23)))</f>
         <v/>
       </c>
       <c r="W22" s="30">
@@ -2433,7 +2433,7 @@
         <v/>
       </c>
       <c r="AD22" s="30">
-        <f>IF(A22&gt;$B$6+$B$7,$B$13/AA23,IF(A22&gt;=$B$6,$B$13*$B$15/AA23,($B$13*$B$15+$B$12)/AA23))</f>
+        <f>IF(A22&gt;$B$6+$B$7,$B$13/AA23,IF(A22=$B$6+$B$7,0,IF(A22&gt;=$B$6,$B$13*$B$15/AA23,($B$13*$B$15+$B$12)/AA23)))</f>
         <v/>
       </c>
       <c r="AE22" s="30">
@@ -2498,7 +2498,7 @@
         <v/>
       </c>
       <c r="F23" s="30">
-        <f>IF(A23&gt;$B$6+$B$7,$B$13/C24,IF(A23&gt;=$B$6,$B$13*$B$15/C24,($B$13*$B$15+$B$12)/C24))</f>
+        <f>IF(A23&gt;$B$6+$B$7,$B$13/C24,IF(A23=$B$6+$B$7,0,IF(A23&gt;=$B$6,$B$13*$B$15/C24,($B$13*$B$15+$B$12)/C24)))</f>
         <v/>
       </c>
       <c r="G23" s="30">
@@ -2530,7 +2530,7 @@
         <v/>
       </c>
       <c r="N23" s="30">
-        <f>IF(A23&gt;$B$6+$B$7,$B$13/K24,IF(A23&gt;=$B$6,$B$13*$B$15/K24,($B$13*$B$15+$B$12)/K24))</f>
+        <f>IF(A23&gt;$B$6+$B$7,$B$13/K24,IF(A23=$B$6+$B$7,0,IF(A23&gt;=$B$6,$B$13*$B$15/K24,($B$13*$B$15+$B$12)/K24)))</f>
         <v/>
       </c>
       <c r="O23" s="30">
@@ -2562,7 +2562,7 @@
         <v/>
       </c>
       <c r="V23" s="30">
-        <f>IF(A23&gt;$B$6+$B$7,$B$13/S24,IF(A23&gt;=$B$6,$B$13*$B$15/S24,($B$13*$B$15+$B$12)/S24))</f>
+        <f>IF(A23&gt;$B$6+$B$7,$B$13/S24,IF(A23=$B$6+$B$7,0,IF(A23&gt;=$B$6,$B$13*$B$15/S24,($B$13*$B$15+$B$12)/S24)))</f>
         <v/>
       </c>
       <c r="W23" s="30">
@@ -2594,7 +2594,7 @@
         <v/>
       </c>
       <c r="AD23" s="30">
-        <f>IF(A23&gt;$B$6+$B$7,$B$13/AA24,IF(A23&gt;=$B$6,$B$13*$B$15/AA24,($B$13*$B$15+$B$12)/AA24))</f>
+        <f>IF(A23&gt;$B$6+$B$7,$B$13/AA24,IF(A23=$B$6+$B$7,0,IF(A23&gt;=$B$6,$B$13*$B$15/AA24,($B$13*$B$15+$B$12)/AA24)))</f>
         <v/>
       </c>
       <c r="AE23" s="30">
@@ -2659,7 +2659,7 @@
         <v/>
       </c>
       <c r="F24" s="30">
-        <f>IF(A24&gt;$B$6+$B$7,$B$13/C25,IF(A24&gt;=$B$6,$B$13*$B$15/C25,($B$13*$B$15+$B$12)/C25))</f>
+        <f>IF(A24&gt;$B$6+$B$7,$B$13/C25,IF(A24=$B$6+$B$7,0,IF(A24&gt;=$B$6,$B$13*$B$15/C25,($B$13*$B$15+$B$12)/C25)))</f>
         <v/>
       </c>
       <c r="G24" s="30">
@@ -2691,7 +2691,7 @@
         <v/>
       </c>
       <c r="N24" s="30">
-        <f>IF(A24&gt;$B$6+$B$7,$B$13/K25,IF(A24&gt;=$B$6,$B$13*$B$15/K25,($B$13*$B$15+$B$12)/K25))</f>
+        <f>IF(A24&gt;$B$6+$B$7,$B$13/K25,IF(A24=$B$6+$B$7,0,IF(A24&gt;=$B$6,$B$13*$B$15/K25,($B$13*$B$15+$B$12)/K25)))</f>
         <v/>
       </c>
       <c r="O24" s="30">
@@ -2723,7 +2723,7 @@
         <v/>
       </c>
       <c r="V24" s="30">
-        <f>IF(A24&gt;$B$6+$B$7,$B$13/S25,IF(A24&gt;=$B$6,$B$13*$B$15/S25,($B$13*$B$15+$B$12)/S25))</f>
+        <f>IF(A24&gt;$B$6+$B$7,$B$13/S25,IF(A24=$B$6+$B$7,0,IF(A24&gt;=$B$6,$B$13*$B$15/S25,($B$13*$B$15+$B$12)/S25)))</f>
         <v/>
       </c>
       <c r="W24" s="30">
@@ -2755,7 +2755,7 @@
         <v/>
       </c>
       <c r="AD24" s="30">
-        <f>IF(A24&gt;$B$6+$B$7,$B$13/AA25,IF(A24&gt;=$B$6,$B$13*$B$15/AA25,($B$13*$B$15+$B$12)/AA25))</f>
+        <f>IF(A24&gt;$B$6+$B$7,$B$13/AA25,IF(A24=$B$6+$B$7,0,IF(A24&gt;=$B$6,$B$13*$B$15/AA25,($B$13*$B$15+$B$12)/AA25)))</f>
         <v/>
       </c>
       <c r="AE24" s="30">
@@ -2820,7 +2820,7 @@
         <v/>
       </c>
       <c r="F25" s="30">
-        <f>IF(A25&gt;$B$6+$B$7,$B$13/C26,IF(A25&gt;=$B$6,$B$13*$B$15/C26,($B$13*$B$15+$B$12)/C26))</f>
+        <f>IF(A25&gt;$B$6+$B$7,$B$13/C26,IF(A25=$B$6+$B$7,0,IF(A25&gt;=$B$6,$B$13*$B$15/C26,($B$13*$B$15+$B$12)/C26)))</f>
         <v/>
       </c>
       <c r="G25" s="30">
@@ -2852,7 +2852,7 @@
         <v/>
       </c>
       <c r="N25" s="30">
-        <f>IF(A25&gt;$B$6+$B$7,$B$13/K26,IF(A25&gt;=$B$6,$B$13*$B$15/K26,($B$13*$B$15+$B$12)/K26))</f>
+        <f>IF(A25&gt;$B$6+$B$7,$B$13/K26,IF(A25=$B$6+$B$7,0,IF(A25&gt;=$B$6,$B$13*$B$15/K26,($B$13*$B$15+$B$12)/K26)))</f>
         <v/>
       </c>
       <c r="O25" s="30">
@@ -2884,7 +2884,7 @@
         <v/>
       </c>
       <c r="V25" s="30">
-        <f>IF(A25&gt;$B$6+$B$7,$B$13/S26,IF(A25&gt;=$B$6,$B$13*$B$15/S26,($B$13*$B$15+$B$12)/S26))</f>
+        <f>IF(A25&gt;$B$6+$B$7,$B$13/S26,IF(A25=$B$6+$B$7,0,IF(A25&gt;=$B$6,$B$13*$B$15/S26,($B$13*$B$15+$B$12)/S26)))</f>
         <v/>
       </c>
       <c r="W25" s="30">
@@ -2916,7 +2916,7 @@
         <v/>
       </c>
       <c r="AD25" s="30">
-        <f>IF(A25&gt;$B$6+$B$7,$B$13/AA26,IF(A25&gt;=$B$6,$B$13*$B$15/AA26,($B$13*$B$15+$B$12)/AA26))</f>
+        <f>IF(A25&gt;$B$6+$B$7,$B$13/AA26,IF(A25=$B$6+$B$7,0,IF(A25&gt;=$B$6,$B$13*$B$15/AA26,($B$13*$B$15+$B$12)/AA26)))</f>
         <v/>
       </c>
       <c r="AE25" s="30">
@@ -2981,7 +2981,7 @@
         <v/>
       </c>
       <c r="F26" s="30">
-        <f>IF(A26&gt;$B$6+$B$7,$B$13/C27,IF(A26&gt;=$B$6,$B$13*$B$15/C27,($B$13*$B$15+$B$12)/C27))</f>
+        <f>IF(A26&gt;$B$6+$B$7,$B$13/C27,IF(A26=$B$6+$B$7,0,IF(A26&gt;=$B$6,$B$13*$B$15/C27,($B$13*$B$15+$B$12)/C27)))</f>
         <v/>
       </c>
       <c r="G26" s="30">
@@ -3013,7 +3013,7 @@
         <v/>
       </c>
       <c r="N26" s="30">
-        <f>IF(A26&gt;$B$6+$B$7,$B$13/K27,IF(A26&gt;=$B$6,$B$13*$B$15/K27,($B$13*$B$15+$B$12)/K27))</f>
+        <f>IF(A26&gt;$B$6+$B$7,$B$13/K27,IF(A26=$B$6+$B$7,0,IF(A26&gt;=$B$6,$B$13*$B$15/K27,($B$13*$B$15+$B$12)/K27)))</f>
         <v/>
       </c>
       <c r="O26" s="30">
@@ -3045,7 +3045,7 @@
         <v/>
       </c>
       <c r="V26" s="30">
-        <f>IF(A26&gt;$B$6+$B$7,$B$13/S27,IF(A26&gt;=$B$6,$B$13*$B$15/S27,($B$13*$B$15+$B$12)/S27))</f>
+        <f>IF(A26&gt;$B$6+$B$7,$B$13/S27,IF(A26=$B$6+$B$7,0,IF(A26&gt;=$B$6,$B$13*$B$15/S27,($B$13*$B$15+$B$12)/S27)))</f>
         <v/>
       </c>
       <c r="W26" s="30">
@@ -3077,7 +3077,7 @@
         <v/>
       </c>
       <c r="AD26" s="30">
-        <f>IF(A26&gt;$B$6+$B$7,$B$13/AA27,IF(A26&gt;=$B$6,$B$13*$B$15/AA27,($B$13*$B$15+$B$12)/AA27))</f>
+        <f>IF(A26&gt;$B$6+$B$7,$B$13/AA27,IF(A26=$B$6+$B$7,0,IF(A26&gt;=$B$6,$B$13*$B$15/AA27,($B$13*$B$15+$B$12)/AA27)))</f>
         <v/>
       </c>
       <c r="AE26" s="30">
@@ -3142,7 +3142,7 @@
         <v/>
       </c>
       <c r="F27" s="30">
-        <f>IF(A27&gt;$B$6+$B$7,$B$13/C28,IF(A27&gt;=$B$6,$B$13*$B$15/C28,($B$13*$B$15+$B$12)/C28))</f>
+        <f>IF(A27&gt;$B$6+$B$7,$B$13/C28,IF(A27=$B$6+$B$7,0,IF(A27&gt;=$B$6,$B$13*$B$15/C28,($B$13*$B$15+$B$12)/C28)))</f>
         <v/>
       </c>
       <c r="G27" s="30">
@@ -3174,7 +3174,7 @@
         <v/>
       </c>
       <c r="N27" s="30">
-        <f>IF(A27&gt;$B$6+$B$7,$B$13/K28,IF(A27&gt;=$B$6,$B$13*$B$15/K28,($B$13*$B$15+$B$12)/K28))</f>
+        <f>IF(A27&gt;$B$6+$B$7,$B$13/K28,IF(A27=$B$6+$B$7,0,IF(A27&gt;=$B$6,$B$13*$B$15/K28,($B$13*$B$15+$B$12)/K28)))</f>
         <v/>
       </c>
       <c r="O27" s="30">
@@ -3206,7 +3206,7 @@
         <v/>
       </c>
       <c r="V27" s="30">
-        <f>IF(A27&gt;$B$6+$B$7,$B$13/S28,IF(A27&gt;=$B$6,$B$13*$B$15/S28,($B$13*$B$15+$B$12)/S28))</f>
+        <f>IF(A27&gt;$B$6+$B$7,$B$13/S28,IF(A27=$B$6+$B$7,0,IF(A27&gt;=$B$6,$B$13*$B$15/S28,($B$13*$B$15+$B$12)/S28)))</f>
         <v/>
       </c>
       <c r="W27" s="30">
@@ -3238,7 +3238,7 @@
         <v/>
       </c>
       <c r="AD27" s="30">
-        <f>IF(A27&gt;$B$6+$B$7,$B$13/AA28,IF(A27&gt;=$B$6,$B$13*$B$15/AA28,($B$13*$B$15+$B$12)/AA28))</f>
+        <f>IF(A27&gt;$B$6+$B$7,$B$13/AA28,IF(A27=$B$6+$B$7,0,IF(A27&gt;=$B$6,$B$13*$B$15/AA28,($B$13*$B$15+$B$12)/AA28)))</f>
         <v/>
       </c>
       <c r="AE27" s="30">
@@ -3303,7 +3303,7 @@
         <v/>
       </c>
       <c r="F28" s="30">
-        <f>IF(A28&gt;$B$6+$B$7,$B$13/C29,IF(A28&gt;=$B$6,$B$13*$B$15/C29,($B$13*$B$15+$B$12)/C29))</f>
+        <f>IF(A28&gt;$B$6+$B$7,$B$13/C29,IF(A28=$B$6+$B$7,0,IF(A28&gt;=$B$6,$B$13*$B$15/C29,($B$13*$B$15+$B$12)/C29)))</f>
         <v/>
       </c>
       <c r="G28" s="30">
@@ -3335,7 +3335,7 @@
         <v/>
       </c>
       <c r="N28" s="30">
-        <f>IF(A28&gt;$B$6+$B$7,$B$13/K29,IF(A28&gt;=$B$6,$B$13*$B$15/K29,($B$13*$B$15+$B$12)/K29))</f>
+        <f>IF(A28&gt;$B$6+$B$7,$B$13/K29,IF(A28=$B$6+$B$7,0,IF(A28&gt;=$B$6,$B$13*$B$15/K29,($B$13*$B$15+$B$12)/K29)))</f>
         <v/>
       </c>
       <c r="O28" s="30">
@@ -3367,7 +3367,7 @@
         <v/>
       </c>
       <c r="V28" s="30">
-        <f>IF(A28&gt;$B$6+$B$7,$B$13/S29,IF(A28&gt;=$B$6,$B$13*$B$15/S29,($B$13*$B$15+$B$12)/S29))</f>
+        <f>IF(A28&gt;$B$6+$B$7,$B$13/S29,IF(A28=$B$6+$B$7,0,IF(A28&gt;=$B$6,$B$13*$B$15/S29,($B$13*$B$15+$B$12)/S29)))</f>
         <v/>
       </c>
       <c r="W28" s="30">
@@ -3399,7 +3399,7 @@
         <v/>
       </c>
       <c r="AD28" s="30">
-        <f>IF(A28&gt;$B$6+$B$7,$B$13/AA29,IF(A28&gt;=$B$6,$B$13*$B$15/AA29,($B$13*$B$15+$B$12)/AA29))</f>
+        <f>IF(A28&gt;$B$6+$B$7,$B$13/AA29,IF(A28=$B$6+$B$7,0,IF(A28&gt;=$B$6,$B$13*$B$15/AA29,($B$13*$B$15+$B$12)/AA29)))</f>
         <v/>
       </c>
       <c r="AE28" s="30">
@@ -3464,7 +3464,7 @@
         <v/>
       </c>
       <c r="F29" s="30">
-        <f>IF(A29&gt;$B$6+$B$7,$B$13/C30,IF(A29&gt;=$B$6,$B$13*$B$15/C30,($B$13*$B$15+$B$12)/C30))</f>
+        <f>IF(A29&gt;$B$6+$B$7,$B$13/C30,IF(A29=$B$6+$B$7,0,IF(A29&gt;=$B$6,$B$13*$B$15/C30,($B$13*$B$15+$B$12)/C30)))</f>
         <v/>
       </c>
       <c r="G29" s="30">
@@ -3496,7 +3496,7 @@
         <v/>
       </c>
       <c r="N29" s="30">
-        <f>IF(A29&gt;$B$6+$B$7,$B$13/K30,IF(A29&gt;=$B$6,$B$13*$B$15/K30,($B$13*$B$15+$B$12)/K30))</f>
+        <f>IF(A29&gt;$B$6+$B$7,$B$13/K30,IF(A29=$B$6+$B$7,0,IF(A29&gt;=$B$6,$B$13*$B$15/K30,($B$13*$B$15+$B$12)/K30)))</f>
         <v/>
       </c>
       <c r="O29" s="30">
@@ -3528,7 +3528,7 @@
         <v/>
       </c>
       <c r="V29" s="30">
-        <f>IF(A29&gt;$B$6+$B$7,$B$13/S30,IF(A29&gt;=$B$6,$B$13*$B$15/S30,($B$13*$B$15+$B$12)/S30))</f>
+        <f>IF(A29&gt;$B$6+$B$7,$B$13/S30,IF(A29=$B$6+$B$7,0,IF(A29&gt;=$B$6,$B$13*$B$15/S30,($B$13*$B$15+$B$12)/S30)))</f>
         <v/>
       </c>
       <c r="W29" s="30">
@@ -3560,7 +3560,7 @@
         <v/>
       </c>
       <c r="AD29" s="30">
-        <f>IF(A29&gt;$B$6+$B$7,$B$13/AA30,IF(A29&gt;=$B$6,$B$13*$B$15/AA30,($B$13*$B$15+$B$12)/AA30))</f>
+        <f>IF(A29&gt;$B$6+$B$7,$B$13/AA30,IF(A29=$B$6+$B$7,0,IF(A29&gt;=$B$6,$B$13*$B$15/AA30,($B$13*$B$15+$B$12)/AA30)))</f>
         <v/>
       </c>
       <c r="AE29" s="30">
@@ -3625,7 +3625,7 @@
         <v/>
       </c>
       <c r="F30" s="30">
-        <f>IF(A30&gt;$B$6+$B$7,$B$13/C31,IF(A30&gt;=$B$6,$B$13*$B$15/C31,($B$13*$B$15+$B$12)/C31))</f>
+        <f>IF(A30&gt;$B$6+$B$7,$B$13/C31,IF(A30=$B$6+$B$7,0,IF(A30&gt;=$B$6,$B$13*$B$15/C31,($B$13*$B$15+$B$12)/C31)))</f>
         <v/>
       </c>
       <c r="G30" s="30">
@@ -3657,7 +3657,7 @@
         <v/>
       </c>
       <c r="N30" s="30">
-        <f>IF(A30&gt;$B$6+$B$7,$B$13/K31,IF(A30&gt;=$B$6,$B$13*$B$15/K31,($B$13*$B$15+$B$12)/K31))</f>
+        <f>IF(A30&gt;$B$6+$B$7,$B$13/K31,IF(A30=$B$6+$B$7,0,IF(A30&gt;=$B$6,$B$13*$B$15/K31,($B$13*$B$15+$B$12)/K31)))</f>
         <v/>
       </c>
       <c r="O30" s="30">
@@ -3689,7 +3689,7 @@
         <v/>
       </c>
       <c r="V30" s="30">
-        <f>IF(A30&gt;$B$6+$B$7,$B$13/S31,IF(A30&gt;=$B$6,$B$13*$B$15/S31,($B$13*$B$15+$B$12)/S31))</f>
+        <f>IF(A30&gt;$B$6+$B$7,$B$13/S31,IF(A30=$B$6+$B$7,0,IF(A30&gt;=$B$6,$B$13*$B$15/S31,($B$13*$B$15+$B$12)/S31)))</f>
         <v/>
       </c>
       <c r="W30" s="30">
@@ -3721,7 +3721,7 @@
         <v/>
       </c>
       <c r="AD30" s="30">
-        <f>IF(A30&gt;$B$6+$B$7,$B$13/AA31,IF(A30&gt;=$B$6,$B$13*$B$15/AA31,($B$13*$B$15+$B$12)/AA31))</f>
+        <f>IF(A30&gt;$B$6+$B$7,$B$13/AA31,IF(A30=$B$6+$B$7,0,IF(A30&gt;=$B$6,$B$13*$B$15/AA31,($B$13*$B$15+$B$12)/AA31)))</f>
         <v/>
       </c>
       <c r="AE30" s="30">
@@ -3786,7 +3786,7 @@
         <v/>
       </c>
       <c r="F31" s="30">
-        <f>IF(A31&gt;$B$6+$B$7,$B$13/C32,IF(A31&gt;=$B$6,$B$13*$B$15/C32,($B$13*$B$15+$B$12)/C32))</f>
+        <f>IF(A31&gt;$B$6+$B$7,$B$13/C32,IF(A31=$B$6+$B$7,0,IF(A31&gt;=$B$6,$B$13*$B$15/C32,($B$13*$B$15+$B$12)/C32)))</f>
         <v/>
       </c>
       <c r="G31" s="30">
@@ -3818,7 +3818,7 @@
         <v/>
       </c>
       <c r="N31" s="30">
-        <f>IF(A31&gt;$B$6+$B$7,$B$13/K32,IF(A31&gt;=$B$6,$B$13*$B$15/K32,($B$13*$B$15+$B$12)/K32))</f>
+        <f>IF(A31&gt;$B$6+$B$7,$B$13/K32,IF(A31=$B$6+$B$7,0,IF(A31&gt;=$B$6,$B$13*$B$15/K32,($B$13*$B$15+$B$12)/K32)))</f>
         <v/>
       </c>
       <c r="O31" s="30">
@@ -3850,7 +3850,7 @@
         <v/>
       </c>
       <c r="V31" s="30">
-        <f>IF(A31&gt;$B$6+$B$7,$B$13/S32,IF(A31&gt;=$B$6,$B$13*$B$15/S32,($B$13*$B$15+$B$12)/S32))</f>
+        <f>IF(A31&gt;$B$6+$B$7,$B$13/S32,IF(A31=$B$6+$B$7,0,IF(A31&gt;=$B$6,$B$13*$B$15/S32,($B$13*$B$15+$B$12)/S32)))</f>
         <v/>
       </c>
       <c r="W31" s="30">
@@ -3882,7 +3882,7 @@
         <v/>
       </c>
       <c r="AD31" s="30">
-        <f>IF(A31&gt;$B$6+$B$7,$B$13/AA32,IF(A31&gt;=$B$6,$B$13*$B$15/AA32,($B$13*$B$15+$B$12)/AA32))</f>
+        <f>IF(A31&gt;$B$6+$B$7,$B$13/AA32,IF(A31=$B$6+$B$7,0,IF(A31&gt;=$B$6,$B$13*$B$15/AA32,($B$13*$B$15+$B$12)/AA32)))</f>
         <v/>
       </c>
       <c r="AE31" s="30">
@@ -3947,7 +3947,7 @@
         <v/>
       </c>
       <c r="F32" s="30">
-        <f>IF(A32&gt;$B$6+$B$7,$B$13/C33,IF(A32&gt;=$B$6,$B$13*$B$15/C33,($B$13*$B$15+$B$12)/C33))</f>
+        <f>IF(A32&gt;$B$6+$B$7,$B$13/C33,IF(A32=$B$6+$B$7,0,IF(A32&gt;=$B$6,$B$13*$B$15/C33,($B$13*$B$15+$B$12)/C33)))</f>
         <v/>
       </c>
       <c r="G32" s="30">
@@ -3979,7 +3979,7 @@
         <v/>
       </c>
       <c r="N32" s="30">
-        <f>IF(A32&gt;$B$6+$B$7,$B$13/K33,IF(A32&gt;=$B$6,$B$13*$B$15/K33,($B$13*$B$15+$B$12)/K33))</f>
+        <f>IF(A32&gt;$B$6+$B$7,$B$13/K33,IF(A32=$B$6+$B$7,0,IF(A32&gt;=$B$6,$B$13*$B$15/K33,($B$13*$B$15+$B$12)/K33)))</f>
         <v/>
       </c>
       <c r="O32" s="30">
@@ -4011,7 +4011,7 @@
         <v/>
       </c>
       <c r="V32" s="30">
-        <f>IF(A32&gt;$B$6+$B$7,$B$13/S33,IF(A32&gt;=$B$6,$B$13*$B$15/S33,($B$13*$B$15+$B$12)/S33))</f>
+        <f>IF(A32&gt;$B$6+$B$7,$B$13/S33,IF(A32=$B$6+$B$7,0,IF(A32&gt;=$B$6,$B$13*$B$15/S33,($B$13*$B$15+$B$12)/S33)))</f>
         <v/>
       </c>
       <c r="W32" s="30">
@@ -4043,7 +4043,7 @@
         <v/>
       </c>
       <c r="AD32" s="30">
-        <f>IF(A32&gt;$B$6+$B$7,$B$13/AA33,IF(A32&gt;=$B$6,$B$13*$B$15/AA33,($B$13*$B$15+$B$12)/AA33))</f>
+        <f>IF(A32&gt;$B$6+$B$7,$B$13/AA33,IF(A32=$B$6+$B$7,0,IF(A32&gt;=$B$6,$B$13*$B$15/AA33,($B$13*$B$15+$B$12)/AA33)))</f>
         <v/>
       </c>
       <c r="AE32" s="30">
@@ -4108,7 +4108,7 @@
         <v/>
       </c>
       <c r="F33" s="30">
-        <f>IF(A33&gt;$B$6+$B$7,$B$13/C34,IF(A33&gt;=$B$6,$B$13*$B$15/C34,($B$13*$B$15+$B$12)/C34))</f>
+        <f>IF(A33&gt;$B$6+$B$7,$B$13/C34,IF(A33=$B$6+$B$7,0,IF(A33&gt;=$B$6,$B$13*$B$15/C34,($B$13*$B$15+$B$12)/C34)))</f>
         <v/>
       </c>
       <c r="G33" s="30">
@@ -4140,7 +4140,7 @@
         <v/>
       </c>
       <c r="N33" s="30">
-        <f>IF(A33&gt;$B$6+$B$7,$B$13/K34,IF(A33&gt;=$B$6,$B$13*$B$15/K34,($B$13*$B$15+$B$12)/K34))</f>
+        <f>IF(A33&gt;$B$6+$B$7,$B$13/K34,IF(A33=$B$6+$B$7,0,IF(A33&gt;=$B$6,$B$13*$B$15/K34,($B$13*$B$15+$B$12)/K34)))</f>
         <v/>
       </c>
       <c r="O33" s="30">
@@ -4172,7 +4172,7 @@
         <v/>
       </c>
       <c r="V33" s="30">
-        <f>IF(A33&gt;$B$6+$B$7,$B$13/S34,IF(A33&gt;=$B$6,$B$13*$B$15/S34,($B$13*$B$15+$B$12)/S34))</f>
+        <f>IF(A33&gt;$B$6+$B$7,$B$13/S34,IF(A33=$B$6+$B$7,0,IF(A33&gt;=$B$6,$B$13*$B$15/S34,($B$13*$B$15+$B$12)/S34)))</f>
         <v/>
       </c>
       <c r="W33" s="30">
@@ -4204,7 +4204,7 @@
         <v/>
       </c>
       <c r="AD33" s="30">
-        <f>IF(A33&gt;$B$6+$B$7,$B$13/AA34,IF(A33&gt;=$B$6,$B$13*$B$15/AA34,($B$13*$B$15+$B$12)/AA34))</f>
+        <f>IF(A33&gt;$B$6+$B$7,$B$13/AA34,IF(A33=$B$6+$B$7,0,IF(A33&gt;=$B$6,$B$13*$B$15/AA34,($B$13*$B$15+$B$12)/AA34)))</f>
         <v/>
       </c>
       <c r="AE33" s="30">
@@ -4269,7 +4269,7 @@
         <v/>
       </c>
       <c r="F34" s="30">
-        <f>IF(A34&gt;$B$6+$B$7,$B$13/C35,IF(A34&gt;=$B$6,$B$13*$B$15/C35,($B$13*$B$15+$B$12)/C35))</f>
+        <f>IF(A34&gt;$B$6+$B$7,$B$13/C35,IF(A34=$B$6+$B$7,0,IF(A34&gt;=$B$6,$B$13*$B$15/C35,($B$13*$B$15+$B$12)/C35)))</f>
         <v/>
       </c>
       <c r="G34" s="30">
@@ -4301,7 +4301,7 @@
         <v/>
       </c>
       <c r="N34" s="30">
-        <f>IF(A34&gt;$B$6+$B$7,$B$13/K35,IF(A34&gt;=$B$6,$B$13*$B$15/K35,($B$13*$B$15+$B$12)/K35))</f>
+        <f>IF(A34&gt;$B$6+$B$7,$B$13/K35,IF(A34=$B$6+$B$7,0,IF(A34&gt;=$B$6,$B$13*$B$15/K35,($B$13*$B$15+$B$12)/K35)))</f>
         <v/>
       </c>
       <c r="O34" s="30">
@@ -4333,7 +4333,7 @@
         <v/>
       </c>
       <c r="V34" s="30">
-        <f>IF(A34&gt;$B$6+$B$7,$B$13/S35,IF(A34&gt;=$B$6,$B$13*$B$15/S35,($B$13*$B$15+$B$12)/S35))</f>
+        <f>IF(A34&gt;$B$6+$B$7,$B$13/S35,IF(A34=$B$6+$B$7,0,IF(A34&gt;=$B$6,$B$13*$B$15/S35,($B$13*$B$15+$B$12)/S35)))</f>
         <v/>
       </c>
       <c r="W34" s="30">
@@ -4365,7 +4365,7 @@
         <v/>
       </c>
       <c r="AD34" s="30">
-        <f>IF(A34&gt;$B$6+$B$7,$B$13/AA35,IF(A34&gt;=$B$6,$B$13*$B$15/AA35,($B$13*$B$15+$B$12)/AA35))</f>
+        <f>IF(A34&gt;$B$6+$B$7,$B$13/AA35,IF(A34=$B$6+$B$7,0,IF(A34&gt;=$B$6,$B$13*$B$15/AA35,($B$13*$B$15+$B$12)/AA35)))</f>
         <v/>
       </c>
       <c r="AE34" s="30">
@@ -4430,7 +4430,7 @@
         <v/>
       </c>
       <c r="F35" s="30">
-        <f>IF(A35&gt;$B$6+$B$7,$B$13/C36,IF(A35&gt;=$B$6,$B$13*$B$15/C36,($B$13*$B$15+$B$12)/C36))</f>
+        <f>IF(A35&gt;$B$6+$B$7,$B$13/C36,IF(A35=$B$6+$B$7,0,IF(A35&gt;=$B$6,$B$13*$B$15/C36,($B$13*$B$15+$B$12)/C36)))</f>
         <v/>
       </c>
       <c r="G35" s="30">
@@ -4462,7 +4462,7 @@
         <v/>
       </c>
       <c r="N35" s="30">
-        <f>IF(A35&gt;$B$6+$B$7,$B$13/K36,IF(A35&gt;=$B$6,$B$13*$B$15/K36,($B$13*$B$15+$B$12)/K36))</f>
+        <f>IF(A35&gt;$B$6+$B$7,$B$13/K36,IF(A35=$B$6+$B$7,0,IF(A35&gt;=$B$6,$B$13*$B$15/K36,($B$13*$B$15+$B$12)/K36)))</f>
         <v/>
       </c>
       <c r="O35" s="30">
@@ -4494,7 +4494,7 @@
         <v/>
       </c>
       <c r="V35" s="30">
-        <f>IF(A35&gt;$B$6+$B$7,$B$13/S36,IF(A35&gt;=$B$6,$B$13*$B$15/S36,($B$13*$B$15+$B$12)/S36))</f>
+        <f>IF(A35&gt;$B$6+$B$7,$B$13/S36,IF(A35=$B$6+$B$7,0,IF(A35&gt;=$B$6,$B$13*$B$15/S36,($B$13*$B$15+$B$12)/S36)))</f>
         <v/>
       </c>
       <c r="W35" s="30">
@@ -4526,7 +4526,7 @@
         <v/>
       </c>
       <c r="AD35" s="30">
-        <f>IF(A35&gt;$B$6+$B$7,$B$13/AA36,IF(A35&gt;=$B$6,$B$13*$B$15/AA36,($B$13*$B$15+$B$12)/AA36))</f>
+        <f>IF(A35&gt;$B$6+$B$7,$B$13/AA36,IF(A35=$B$6+$B$7,0,IF(A35&gt;=$B$6,$B$13*$B$15/AA36,($B$13*$B$15+$B$12)/AA36)))</f>
         <v/>
       </c>
       <c r="AE35" s="30">
@@ -4591,7 +4591,7 @@
         <v/>
       </c>
       <c r="F36" s="30">
-        <f>IF(A36&gt;$B$6+$B$7,$B$13/C37,IF(A36&gt;=$B$6,$B$13*$B$15/C37,($B$13*$B$15+$B$12)/C37))</f>
+        <f>IF(A36&gt;$B$6+$B$7,$B$13/C37,IF(A36=$B$6+$B$7,0,IF(A36&gt;=$B$6,$B$13*$B$15/C37,($B$13*$B$15+$B$12)/C37)))</f>
         <v/>
       </c>
       <c r="G36" s="30">
@@ -4623,7 +4623,7 @@
         <v/>
       </c>
       <c r="N36" s="30">
-        <f>IF(A36&gt;$B$6+$B$7,$B$13/K37,IF(A36&gt;=$B$6,$B$13*$B$15/K37,($B$13*$B$15+$B$12)/K37))</f>
+        <f>IF(A36&gt;$B$6+$B$7,$B$13/K37,IF(A36=$B$6+$B$7,0,IF(A36&gt;=$B$6,$B$13*$B$15/K37,($B$13*$B$15+$B$12)/K37)))</f>
         <v/>
       </c>
       <c r="O36" s="30">
@@ -4655,7 +4655,7 @@
         <v/>
       </c>
       <c r="V36" s="30">
-        <f>IF(A36&gt;$B$6+$B$7,$B$13/S37,IF(A36&gt;=$B$6,$B$13*$B$15/S37,($B$13*$B$15+$B$12)/S37))</f>
+        <f>IF(A36&gt;$B$6+$B$7,$B$13/S37,IF(A36=$B$6+$B$7,0,IF(A36&gt;=$B$6,$B$13*$B$15/S37,($B$13*$B$15+$B$12)/S37)))</f>
         <v/>
       </c>
       <c r="W36" s="30">
@@ -4687,7 +4687,7 @@
         <v/>
       </c>
       <c r="AD36" s="30">
-        <f>IF(A36&gt;$B$6+$B$7,$B$13/AA37,IF(A36&gt;=$B$6,$B$13*$B$15/AA37,($B$13*$B$15+$B$12)/AA37))</f>
+        <f>IF(A36&gt;$B$6+$B$7,$B$13/AA37,IF(A36=$B$6+$B$7,0,IF(A36&gt;=$B$6,$B$13*$B$15/AA37,($B$13*$B$15+$B$12)/AA37)))</f>
         <v/>
       </c>
       <c r="AE36" s="30">
@@ -4752,7 +4752,7 @@
         <v/>
       </c>
       <c r="F37" s="30">
-        <f>IF(A37&gt;$B$6+$B$7,$B$13/C38,IF(A37&gt;=$B$6,$B$13*$B$15/C38,($B$13*$B$15+$B$12)/C38))</f>
+        <f>IF(A37&gt;$B$6+$B$7,$B$13/C38,IF(A37=$B$6+$B$7,0,IF(A37&gt;=$B$6,$B$13*$B$15/C38,($B$13*$B$15+$B$12)/C38)))</f>
         <v/>
       </c>
       <c r="G37" s="30">
@@ -4784,7 +4784,7 @@
         <v/>
       </c>
       <c r="N37" s="30">
-        <f>IF(A37&gt;$B$6+$B$7,$B$13/K38,IF(A37&gt;=$B$6,$B$13*$B$15/K38,($B$13*$B$15+$B$12)/K38))</f>
+        <f>IF(A37&gt;$B$6+$B$7,$B$13/K38,IF(A37=$B$6+$B$7,0,IF(A37&gt;=$B$6,$B$13*$B$15/K38,($B$13*$B$15+$B$12)/K38)))</f>
         <v/>
       </c>
       <c r="O37" s="30">
@@ -4816,7 +4816,7 @@
         <v/>
       </c>
       <c r="V37" s="30">
-        <f>IF(A37&gt;$B$6+$B$7,$B$13/S38,IF(A37&gt;=$B$6,$B$13*$B$15/S38,($B$13*$B$15+$B$12)/S38))</f>
+        <f>IF(A37&gt;$B$6+$B$7,$B$13/S38,IF(A37=$B$6+$B$7,0,IF(A37&gt;=$B$6,$B$13*$B$15/S38,($B$13*$B$15+$B$12)/S38)))</f>
         <v/>
       </c>
       <c r="W37" s="30">
@@ -4848,7 +4848,7 @@
         <v/>
       </c>
       <c r="AD37" s="30">
-        <f>IF(A37&gt;$B$6+$B$7,$B$13/AA38,IF(A37&gt;=$B$6,$B$13*$B$15/AA38,($B$13*$B$15+$B$12)/AA38))</f>
+        <f>IF(A37&gt;$B$6+$B$7,$B$13/AA38,IF(A37=$B$6+$B$7,0,IF(A37&gt;=$B$6,$B$13*$B$15/AA38,($B$13*$B$15+$B$12)/AA38)))</f>
         <v/>
       </c>
       <c r="AE37" s="30">
@@ -4913,7 +4913,7 @@
         <v/>
       </c>
       <c r="F38" s="30">
-        <f>IF(A38&gt;$B$6+$B$7,$B$13/C39,IF(A38&gt;=$B$6,$B$13*$B$15/C39,($B$13*$B$15+$B$12)/C39))</f>
+        <f>IF(A38&gt;$B$6+$B$7,$B$13/C39,IF(A38=$B$6+$B$7,0,IF(A38&gt;=$B$6,$B$13*$B$15/C39,($B$13*$B$15+$B$12)/C39)))</f>
         <v/>
       </c>
       <c r="G38" s="30">
@@ -4945,7 +4945,7 @@
         <v/>
       </c>
       <c r="N38" s="30">
-        <f>IF(A38&gt;$B$6+$B$7,$B$13/K39,IF(A38&gt;=$B$6,$B$13*$B$15/K39,($B$13*$B$15+$B$12)/K39))</f>
+        <f>IF(A38&gt;$B$6+$B$7,$B$13/K39,IF(A38=$B$6+$B$7,0,IF(A38&gt;=$B$6,$B$13*$B$15/K39,($B$13*$B$15+$B$12)/K39)))</f>
         <v/>
       </c>
       <c r="O38" s="30">
@@ -4977,7 +4977,7 @@
         <v/>
       </c>
       <c r="V38" s="30">
-        <f>IF(A38&gt;$B$6+$B$7,$B$13/S39,IF(A38&gt;=$B$6,$B$13*$B$15/S39,($B$13*$B$15+$B$12)/S39))</f>
+        <f>IF(A38&gt;$B$6+$B$7,$B$13/S39,IF(A38=$B$6+$B$7,0,IF(A38&gt;=$B$6,$B$13*$B$15/S39,($B$13*$B$15+$B$12)/S39)))</f>
         <v/>
       </c>
       <c r="W38" s="30">
@@ -5009,7 +5009,7 @@
         <v/>
       </c>
       <c r="AD38" s="30">
-        <f>IF(A38&gt;$B$6+$B$7,$B$13/AA39,IF(A38&gt;=$B$6,$B$13*$B$15/AA39,($B$13*$B$15+$B$12)/AA39))</f>
+        <f>IF(A38&gt;$B$6+$B$7,$B$13/AA39,IF(A38=$B$6+$B$7,0,IF(A38&gt;=$B$6,$B$13*$B$15/AA39,($B$13*$B$15+$B$12)/AA39)))</f>
         <v/>
       </c>
       <c r="AE38" s="30">
@@ -5074,7 +5074,7 @@
         <v/>
       </c>
       <c r="F39" s="30">
-        <f>IF(A39&gt;$B$6+$B$7,$B$13/C40,IF(A39&gt;=$B$6,$B$13*$B$15/C40,($B$13*$B$15+$B$12)/C40))</f>
+        <f>IF(A39&gt;$B$6+$B$7,$B$13/C40,IF(A39=$B$6+$B$7,0,IF(A39&gt;=$B$6,$B$13*$B$15/C40,($B$13*$B$15+$B$12)/C40)))</f>
         <v/>
       </c>
       <c r="G39" s="30">
@@ -5106,7 +5106,7 @@
         <v/>
       </c>
       <c r="N39" s="30">
-        <f>IF(A39&gt;$B$6+$B$7,$B$13/K40,IF(A39&gt;=$B$6,$B$13*$B$15/K40,($B$13*$B$15+$B$12)/K40))</f>
+        <f>IF(A39&gt;$B$6+$B$7,$B$13/K40,IF(A39=$B$6+$B$7,0,IF(A39&gt;=$B$6,$B$13*$B$15/K40,($B$13*$B$15+$B$12)/K40)))</f>
         <v/>
       </c>
       <c r="O39" s="30">
@@ -5138,7 +5138,7 @@
         <v/>
       </c>
       <c r="V39" s="30">
-        <f>IF(A39&gt;$B$6+$B$7,$B$13/S40,IF(A39&gt;=$B$6,$B$13*$B$15/S40,($B$13*$B$15+$B$12)/S40))</f>
+        <f>IF(A39&gt;$B$6+$B$7,$B$13/S40,IF(A39=$B$6+$B$7,0,IF(A39&gt;=$B$6,$B$13*$B$15/S40,($B$13*$B$15+$B$12)/S40)))</f>
         <v/>
       </c>
       <c r="W39" s="30">
@@ -5170,7 +5170,7 @@
         <v/>
       </c>
       <c r="AD39" s="30">
-        <f>IF(A39&gt;$B$6+$B$7,$B$13/AA40,IF(A39&gt;=$B$6,$B$13*$B$15/AA40,($B$13*$B$15+$B$12)/AA40))</f>
+        <f>IF(A39&gt;$B$6+$B$7,$B$13/AA40,IF(A39=$B$6+$B$7,0,IF(A39&gt;=$B$6,$B$13*$B$15/AA40,($B$13*$B$15+$B$12)/AA40)))</f>
         <v/>
       </c>
       <c r="AE39" s="30">
@@ -5235,7 +5235,7 @@
         <v/>
       </c>
       <c r="F40" s="30">
-        <f>IF(A40&gt;$B$6+$B$7,$B$13/C41,IF(A40&gt;=$B$6,$B$13*$B$15/C41,($B$13*$B$15+$B$12)/C41))</f>
+        <f>IF(A40&gt;$B$6+$B$7,$B$13/C41,IF(A40=$B$6+$B$7,0,IF(A40&gt;=$B$6,$B$13*$B$15/C41,($B$13*$B$15+$B$12)/C41)))</f>
         <v/>
       </c>
       <c r="G40" s="30">
@@ -5267,7 +5267,7 @@
         <v/>
       </c>
       <c r="N40" s="30">
-        <f>IF(A40&gt;$B$6+$B$7,$B$13/K41,IF(A40&gt;=$B$6,$B$13*$B$15/K41,($B$13*$B$15+$B$12)/K41))</f>
+        <f>IF(A40&gt;$B$6+$B$7,$B$13/K41,IF(A40=$B$6+$B$7,0,IF(A40&gt;=$B$6,$B$13*$B$15/K41,($B$13*$B$15+$B$12)/K41)))</f>
         <v/>
       </c>
       <c r="O40" s="30">
@@ -5299,7 +5299,7 @@
         <v/>
       </c>
       <c r="V40" s="30">
-        <f>IF(A40&gt;$B$6+$B$7,$B$13/S41,IF(A40&gt;=$B$6,$B$13*$B$15/S41,($B$13*$B$15+$B$12)/S41))</f>
+        <f>IF(A40&gt;$B$6+$B$7,$B$13/S41,IF(A40=$B$6+$B$7,0,IF(A40&gt;=$B$6,$B$13*$B$15/S41,($B$13*$B$15+$B$12)/S41)))</f>
         <v/>
       </c>
       <c r="W40" s="30">
@@ -5331,7 +5331,7 @@
         <v/>
       </c>
       <c r="AD40" s="30">
-        <f>IF(A40&gt;$B$6+$B$7,$B$13/AA41,IF(A40&gt;=$B$6,$B$13*$B$15/AA41,($B$13*$B$15+$B$12)/AA41))</f>
+        <f>IF(A40&gt;$B$6+$B$7,$B$13/AA41,IF(A40=$B$6+$B$7,0,IF(A40&gt;=$B$6,$B$13*$B$15/AA41,($B$13*$B$15+$B$12)/AA41)))</f>
         <v/>
       </c>
       <c r="AE40" s="30">
@@ -5396,7 +5396,7 @@
         <v/>
       </c>
       <c r="F41" s="30">
-        <f>IF(A41&gt;$B$6+$B$7,$B$13/C42,IF(A41&gt;=$B$6,$B$13*$B$15/C42,($B$13*$B$15+$B$12)/C42))</f>
+        <f>IF(A41&gt;$B$6+$B$7,$B$13/C42,IF(A41=$B$6+$B$7,0,IF(A41&gt;=$B$6,$B$13*$B$15/C42,($B$13*$B$15+$B$12)/C42)))</f>
         <v/>
       </c>
       <c r="G41" s="30">
@@ -5428,7 +5428,7 @@
         <v/>
       </c>
       <c r="N41" s="30">
-        <f>IF(A41&gt;$B$6+$B$7,$B$13/K42,IF(A41&gt;=$B$6,$B$13*$B$15/K42,($B$13*$B$15+$B$12)/K42))</f>
+        <f>IF(A41&gt;$B$6+$B$7,$B$13/K42,IF(A41=$B$6+$B$7,0,IF(A41&gt;=$B$6,$B$13*$B$15/K42,($B$13*$B$15+$B$12)/K42)))</f>
         <v/>
       </c>
       <c r="O41" s="30">
@@ -5460,7 +5460,7 @@
         <v/>
       </c>
       <c r="V41" s="30">
-        <f>IF(A41&gt;$B$6+$B$7,$B$13/S42,IF(A41&gt;=$B$6,$B$13*$B$15/S42,($B$13*$B$15+$B$12)/S42))</f>
+        <f>IF(A41&gt;$B$6+$B$7,$B$13/S42,IF(A41=$B$6+$B$7,0,IF(A41&gt;=$B$6,$B$13*$B$15/S42,($B$13*$B$15+$B$12)/S42)))</f>
         <v/>
       </c>
       <c r="W41" s="30">
@@ -5492,7 +5492,7 @@
         <v/>
       </c>
       <c r="AD41" s="30">
-        <f>IF(A41&gt;$B$6+$B$7,$B$13/AA42,IF(A41&gt;=$B$6,$B$13*$B$15/AA42,($B$13*$B$15+$B$12)/AA42))</f>
+        <f>IF(A41&gt;$B$6+$B$7,$B$13/AA42,IF(A41=$B$6+$B$7,0,IF(A41&gt;=$B$6,$B$13*$B$15/AA42,($B$13*$B$15+$B$12)/AA42)))</f>
         <v/>
       </c>
       <c r="AE41" s="30">
@@ -5557,7 +5557,7 @@
         <v/>
       </c>
       <c r="F42" s="30">
-        <f>IF(A42&gt;$B$6+$B$7,$B$13/C43,IF(A42&gt;=$B$6,$B$13*$B$15/C43,($B$13*$B$15+$B$12)/C43))</f>
+        <f>IF(A42&gt;$B$6+$B$7,$B$13/C43,IF(A42=$B$6+$B$7,0,IF(A42&gt;=$B$6,$B$13*$B$15/C43,($B$13*$B$15+$B$12)/C43)))</f>
         <v/>
       </c>
       <c r="G42" s="30">
@@ -5589,7 +5589,7 @@
         <v/>
       </c>
       <c r="N42" s="30">
-        <f>IF(A42&gt;$B$6+$B$7,$B$13/K43,IF(A42&gt;=$B$6,$B$13*$B$15/K43,($B$13*$B$15+$B$12)/K43))</f>
+        <f>IF(A42&gt;$B$6+$B$7,$B$13/K43,IF(A42=$B$6+$B$7,0,IF(A42&gt;=$B$6,$B$13*$B$15/K43,($B$13*$B$15+$B$12)/K43)))</f>
         <v/>
       </c>
       <c r="O42" s="30">
@@ -5621,7 +5621,7 @@
         <v/>
       </c>
       <c r="V42" s="30">
-        <f>IF(A42&gt;$B$6+$B$7,$B$13/S43,IF(A42&gt;=$B$6,$B$13*$B$15/S43,($B$13*$B$15+$B$12)/S43))</f>
+        <f>IF(A42&gt;$B$6+$B$7,$B$13/S43,IF(A42=$B$6+$B$7,0,IF(A42&gt;=$B$6,$B$13*$B$15/S43,($B$13*$B$15+$B$12)/S43)))</f>
         <v/>
       </c>
       <c r="W42" s="30">
@@ -5653,7 +5653,7 @@
         <v/>
       </c>
       <c r="AD42" s="30">
-        <f>IF(A42&gt;$B$6+$B$7,$B$13/AA43,IF(A42&gt;=$B$6,$B$13*$B$15/AA43,($B$13*$B$15+$B$12)/AA43))</f>
+        <f>IF(A42&gt;$B$6+$B$7,$B$13/AA43,IF(A42=$B$6+$B$7,0,IF(A42&gt;=$B$6,$B$13*$B$15/AA43,($B$13*$B$15+$B$12)/AA43)))</f>
         <v/>
       </c>
       <c r="AE42" s="30">
@@ -5718,7 +5718,7 @@
         <v/>
       </c>
       <c r="F43" s="30">
-        <f>IF(A43&gt;$B$6+$B$7,$B$13/C44,IF(A43&gt;=$B$6,$B$13*$B$15/C44,($B$13*$B$15+$B$12)/C44))</f>
+        <f>IF(A43&gt;$B$6+$B$7,$B$13/C44,IF(A43=$B$6+$B$7,0,IF(A43&gt;=$B$6,$B$13*$B$15/C44,($B$13*$B$15+$B$12)/C44)))</f>
         <v/>
       </c>
       <c r="G43" s="30">
@@ -5750,7 +5750,7 @@
         <v/>
       </c>
       <c r="N43" s="30">
-        <f>IF(A43&gt;$B$6+$B$7,$B$13/K44,IF(A43&gt;=$B$6,$B$13*$B$15/K44,($B$13*$B$15+$B$12)/K44))</f>
+        <f>IF(A43&gt;$B$6+$B$7,$B$13/K44,IF(A43=$B$6+$B$7,0,IF(A43&gt;=$B$6,$B$13*$B$15/K44,($B$13*$B$15+$B$12)/K44)))</f>
         <v/>
       </c>
       <c r="O43" s="30">
@@ -5782,7 +5782,7 @@
         <v/>
       </c>
       <c r="V43" s="30">
-        <f>IF(A43&gt;$B$6+$B$7,$B$13/S44,IF(A43&gt;=$B$6,$B$13*$B$15/S44,($B$13*$B$15+$B$12)/S44))</f>
+        <f>IF(A43&gt;$B$6+$B$7,$B$13/S44,IF(A43=$B$6+$B$7,0,IF(A43&gt;=$B$6,$B$13*$B$15/S44,($B$13*$B$15+$B$12)/S44)))</f>
         <v/>
       </c>
       <c r="W43" s="30">
@@ -5814,7 +5814,7 @@
         <v/>
       </c>
       <c r="AD43" s="30">
-        <f>IF(A43&gt;$B$6+$B$7,$B$13/AA44,IF(A43&gt;=$B$6,$B$13*$B$15/AA44,($B$13*$B$15+$B$12)/AA44))</f>
+        <f>IF(A43&gt;$B$6+$B$7,$B$13/AA44,IF(A43=$B$6+$B$7,0,IF(A43&gt;=$B$6,$B$13*$B$15/AA44,($B$13*$B$15+$B$12)/AA44)))</f>
         <v/>
       </c>
       <c r="AE43" s="30">

</xml_diff>